<commit_message>
Mejora de ambiente de prueba, agregados de copi y codigos Ecuador
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
@@ -479,7 +479,7 @@
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="53" customWidth="1" min="9" max="9"/>
+    <col width="58" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -583,7 +583,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15/10/2025</t>
+          <t>24/10/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="I264" s="11" t="inlineStr">
         <is>
-          <t>DEVOLUCION MERCANCI AAAA- DEVOLUCION MERCANCI AAAA-</t>
+          <t>DEV DEVOLUCION MERCANCI AAAA- RANCHO</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="I265" s="11" t="inlineStr">
         <is>
-          <t>DEVOLUCION MERCANCI AAAA- DEVOLUCION MERCANCI AAAA-</t>
+          <t>DEV DEVOLUCION MERCANCI AAAA- PERFUME</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5877,7 @@
       </c>
       <c r="I266" s="11" t="inlineStr">
         <is>
-          <t>DROGUE DEVOLUCIONES</t>
+          <t>DND DSCTO 20.171.100.014.225 DEVOLUCIONES DROGUE</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="I267" s="11" t="inlineStr">
         <is>
-          <t>DROGUE DEVOLUCIONES</t>
+          <t>DND DSCTO 20.181.100.045.651 DEVOLUCIONES DROGUE</t>
         </is>
       </c>
     </row>
@@ -5943,7 +5943,7 @@
       </c>
       <c r="I268" s="11" t="inlineStr">
         <is>
-          <t>DROGUE DSTO COMERCIAL FIJO</t>
+          <t>DCF DSCTO 20.171.100.014.225 DSTO COMERCIAL FIJO DROGUE</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
       </c>
       <c r="I269" s="11" t="inlineStr">
         <is>
-          <t>DROGUE DSTO COMERCIAL FIJO</t>
+          <t>DCF DSCTO 20.181.100.032.054 DSTO COMERCIAL FIJO DROGUE</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6009,7 @@
       </c>
       <c r="I270" s="11" t="inlineStr">
         <is>
-          <t>DROGUE DSTO COMERCIAL FIJO</t>
+          <t>DCF DSCTO 20.181.100.045.651 DSTO COMERCIAL FIJO DROGUE</t>
         </is>
       </c>
     </row>
@@ -6042,7 +6042,7 @@
       </c>
       <c r="I271" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEED VPP2 2020716</t>
+          <t>VPP2 2020716</t>
         </is>
       </c>
     </row>
@@ -6075,7 +6075,7 @@
       </c>
       <c r="I272" s="11" t="inlineStr">
         <is>
-          <t>PERFUME DESCUENTO CALENDARI</t>
+          <t>DCA DSCTO 20.251.200.196.961 DESCUENTO CALENDARI PERFUME</t>
         </is>
       </c>
     </row>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="I273" s="11" t="inlineStr">
         <is>
-          <t>PERFUME DEVOLUCIONES</t>
+          <t>DND DSCTO 20.171.200.014.220 DEVOLUCIONES PERFUME</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="I274" s="11" t="inlineStr">
         <is>
-          <t>PERFUME DSTO COMERCIAL FIJO</t>
+          <t>DCF DSCTO 20.171.200.014.220 DSTO COMERCIAL FIJO PERFUME</t>
         </is>
       </c>
     </row>
@@ -6174,7 +6174,7 @@
       </c>
       <c r="I275" s="11" t="inlineStr">
         <is>
-          <t>PERFUME DSTO COMERCIAL FIJO</t>
+          <t>DCF DSCTO 20.181.200.033.536 DSTO COMERCIAL FIJO PERFUME</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="I276" s="11" t="inlineStr">
         <is>
-          <t>PLATOS DESCUENTO APERTURA</t>
+          <t>DAT DSCTO 20.252.600.197.745 DESCUENTO APERTURA PLATOS</t>
         </is>
       </c>
     </row>
@@ -6240,7 +6240,7 @@
       </c>
       <c r="I277" s="11" t="inlineStr">
         <is>
-          <t>PLATOS DESCUENTO COMPRAS</t>
+          <t>DCC DSCTO 20.222.600.126.372 DESCUENTO COMPRAS PLATOS</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6273,7 @@
       </c>
       <c r="I278" s="11" t="inlineStr">
         <is>
-          <t>PLATOS DSTO COMERCIAL FIJO</t>
+          <t>DCF DSCTO 20.222.600.126.372 DSTO COMERCIAL FIJO PLATOS</t>
         </is>
       </c>
     </row>
@@ -6306,7 +6306,7 @@
       </c>
       <c r="I279" s="11" t="inlineStr">
         <is>
-          <t>RANCHO DESCUENTO</t>
+          <t>RPL DSCTO 0 DESCUENTO RANCHO</t>
         </is>
       </c>
     </row>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="I280" s="11" t="inlineStr">
         <is>
-          <t>RANCHO DESCUENTO CALENDARI</t>
+          <t>DCA DSCTO 20.251.400.197.145 DESCUENTO CALENDARI RANCHO</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="I281" s="11" t="inlineStr">
         <is>
-          <t>RANCHO DESCUENTO CALENDARI</t>
+          <t>DCA DSCTO 20.251.400.197.146 DESCUENTO CALENDARI RANCHO</t>
         </is>
       </c>
     </row>
@@ -6405,7 +6405,7 @@
       </c>
       <c r="I282" s="11" t="inlineStr">
         <is>
-          <t>RANCHO DESCUENTO CALENDARI</t>
+          <t>DCA DSCTO 20.251.400.197.147 DESCUENTO CALENDARI RANCHO</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="I283" s="11" t="inlineStr">
         <is>
-          <t>RANCHO DESCUENTO CALENDARI</t>
+          <t>DCA DSCTO 20.251.400.197.148 DESCUENTO CALENDARI RANCHO</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="I284" s="11" t="inlineStr">
         <is>
-          <t>RANCHO DESCUENTO EN PRIMER</t>
+          <t>DPC DSCTO 0 DESCUENTO EN PRIMER RANCHO</t>
         </is>
       </c>
     </row>
@@ -7362,14 +7362,14 @@
       </c>
       <c r="I311" s="11" t="inlineStr">
         <is>
-          <t>Costo de Transferen Costo de Transferen</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="C312" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D312" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Mejora en codigos de Colombia de filtros parametros id clientes y nro clientes. Y tamnbien se agrego el codigo de Euro, tal cual estaba en Pruebas
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
@@ -543,8 +543,10 @@
           <t>Codigo de Cliente</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
-        <v>10267301</v>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>10267301.0</t>
+        </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cambios en funcion merge
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I482"/>
+  <dimension ref="A1:I483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7969,33 +7969,29 @@
     <row r="368">
       <c r="C368" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Nota de Crédito</t>
         </is>
       </c>
       <c r="D368" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO APERTURA</t>
+          <t>1200016485</t>
         </is>
       </c>
       <c r="E368" s="6" t="n">
-        <v>-8594192</v>
+        <v>-4509059502</v>
       </c>
       <c r="F368" s="10" t="inlineStr">
         <is>
-          <t>DROGUE</t>
-        </is>
-      </c>
-      <c r="G368" s="10" t="inlineStr">
-        <is>
-          <t>987</t>
-        </is>
-      </c>
+          <t>NRO</t>
+        </is>
+      </c>
+      <c r="G368" s="10" t="inlineStr"/>
       <c r="H368" s="6" t="n">
-        <v>-8594192</v>
+        <v>-4509059502</v>
       </c>
       <c r="I368" s="11" t="inlineStr">
         <is>
-          <t>DAV DSCTO  DESCUENTO APERTURA DROGUE</t>
+          <t>favor del cliente sin aplicar por falta de soporte</t>
         </is>
       </c>
     </row>
@@ -8007,11 +8003,11 @@
       </c>
       <c r="D369" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>DESCUENTO APERTURA</t>
         </is>
       </c>
       <c r="E369" s="6" t="n">
-        <v>-817508590</v>
+        <v>-8594192</v>
       </c>
       <c r="F369" s="10" t="inlineStr">
         <is>
@@ -8024,11 +8020,11 @@
         </is>
       </c>
       <c r="H369" s="6" t="n">
-        <v>-817508590</v>
+        <v>-8594192</v>
       </c>
       <c r="I369" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO  DESCUENTO CALENDARI DROGUE</t>
+          <t>DAV DSCTO  DESCUENTO APERTURA DROGUE</t>
         </is>
       </c>
     </row>
@@ -8040,11 +8036,11 @@
       </c>
       <c r="D370" s="10" t="inlineStr">
         <is>
-          <t>DEVOLUCIONES</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E370" s="6" t="n">
-        <v>-3512351</v>
+        <v>-817508590</v>
       </c>
       <c r="F370" s="10" t="inlineStr">
         <is>
@@ -8057,11 +8053,11 @@
         </is>
       </c>
       <c r="H370" s="6" t="n">
-        <v>-3512351</v>
+        <v>-817508590</v>
       </c>
       <c r="I370" s="11" t="inlineStr">
         <is>
-          <t>DND DSCTO  DEVOLUCIONES DROGUE</t>
+          <t>DCA DSCTO  DESCUENTO CALENDARI DROGUE</t>
         </is>
       </c>
     </row>
@@ -8073,11 +8069,11 @@
       </c>
       <c r="D371" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>DEVOLUCIONES</t>
         </is>
       </c>
       <c r="E371" s="6" t="n">
-        <v>-48283208</v>
+        <v>-3512351</v>
       </c>
       <c r="F371" s="10" t="inlineStr">
         <is>
@@ -8090,11 +8086,11 @@
         </is>
       </c>
       <c r="H371" s="6" t="n">
-        <v>-48283208</v>
+        <v>-3512351</v>
       </c>
       <c r="I371" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO  DSTO COMERCIAL FIJO DROGUE</t>
+          <t>DND DSCTO  DEVOLUCIONES DROGUE</t>
         </is>
       </c>
     </row>
@@ -8106,11 +8102,11 @@
       </c>
       <c r="D372" s="10" t="inlineStr">
         <is>
-          <t>DTO POR ESCALA VOLU</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E372" s="6" t="n">
-        <v>-67702329</v>
+        <v>-48283208</v>
       </c>
       <c r="F372" s="10" t="inlineStr">
         <is>
@@ -8123,11 +8119,11 @@
         </is>
       </c>
       <c r="H372" s="6" t="n">
-        <v>-67702329</v>
+        <v>-48283208</v>
       </c>
       <c r="I372" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO  DTO POR ESCALA VOLU DROGUE</t>
+          <t>DCF DSCTO  DSTO COMERCIAL FIJO DROGUE</t>
         </is>
       </c>
     </row>
@@ -8143,7 +8139,7 @@
         </is>
       </c>
       <c r="E373" s="6" t="n">
-        <v>-2165916</v>
+        <v>-67702329</v>
       </c>
       <c r="F373" s="10" t="inlineStr">
         <is>
@@ -8156,11 +8152,11 @@
         </is>
       </c>
       <c r="H373" s="6" t="n">
-        <v>-2165916</v>
+        <v>-67702329</v>
       </c>
       <c r="I373" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20251100199283 DTO POR ESCALA VOLU DROGUE</t>
+          <t>DEC DSCTO  DTO POR ESCALA VOLU DROGUE</t>
         </is>
       </c>
     </row>
@@ -8172,28 +8168,28 @@
       </c>
       <c r="D374" s="10" t="inlineStr">
         <is>
-          <t>VPP1 2004529ADM. FIDELIDAD -</t>
+          <t>DTO POR ESCALA VOLU</t>
         </is>
       </c>
       <c r="E374" s="6" t="n">
-        <v>-57239000</v>
+        <v>-2165916</v>
       </c>
       <c r="F374" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEED</t>
+          <t>DROGUE</t>
         </is>
       </c>
       <c r="G374" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H374" s="6" t="n">
-        <v>-57239000</v>
+        <v>-2165916</v>
       </c>
       <c r="I374" s="11" t="inlineStr">
         <is>
-          <t>VPP1 2004529ADM. FIDELIDAD -</t>
+          <t>DEC DSCTO 20251100199283 DTO POR ESCALA VOLU DROGUE</t>
         </is>
       </c>
     </row>
@@ -8205,11 +8201,11 @@
       </c>
       <c r="D375" s="10" t="inlineStr">
         <is>
-          <t>VPP1 2004621ADM. FIDELIDAD -</t>
+          <t>VPP1 2004529ADM. FIDELIDAD -</t>
         </is>
       </c>
       <c r="E375" s="6" t="n">
-        <v>-6426000</v>
+        <v>-57239000</v>
       </c>
       <c r="F375" s="10" t="inlineStr">
         <is>
@@ -8222,11 +8218,11 @@
         </is>
       </c>
       <c r="H375" s="6" t="n">
-        <v>-6426000</v>
+        <v>-57239000</v>
       </c>
       <c r="I375" s="11" t="inlineStr">
         <is>
-          <t>VPP1 2004621ADM. FIDELIDAD -</t>
+          <t>VPP1 2004529ADM. FIDELIDAD -</t>
         </is>
       </c>
     </row>
@@ -8238,11 +8234,11 @@
       </c>
       <c r="D376" s="10" t="inlineStr">
         <is>
-          <t>VPP1 2004622ADM. FIDELIDAD -</t>
+          <t>VPP1 2004621ADM. FIDELIDAD -</t>
         </is>
       </c>
       <c r="E376" s="6" t="n">
-        <v>-41650000</v>
+        <v>-6426000</v>
       </c>
       <c r="F376" s="10" t="inlineStr">
         <is>
@@ -8255,11 +8251,11 @@
         </is>
       </c>
       <c r="H376" s="6" t="n">
-        <v>-41650000</v>
+        <v>-6426000</v>
       </c>
       <c r="I376" s="11" t="inlineStr">
         <is>
-          <t>VPP1 2004622ADM. FIDELIDAD -</t>
+          <t>VPP1 2004621ADM. FIDELIDAD -</t>
         </is>
       </c>
     </row>
@@ -8271,11 +8267,11 @@
       </c>
       <c r="D377" s="10" t="inlineStr">
         <is>
-          <t>VPP2 2021716ADM.</t>
+          <t>VPP1 2004622ADM. FIDELIDAD -</t>
         </is>
       </c>
       <c r="E377" s="6" t="n">
-        <v>-2507098292</v>
+        <v>-41650000</v>
       </c>
       <c r="F377" s="10" t="inlineStr">
         <is>
@@ -8288,11 +8284,11 @@
         </is>
       </c>
       <c r="H377" s="6" t="n">
-        <v>-2507098292</v>
+        <v>-41650000</v>
       </c>
       <c r="I377" s="11" t="inlineStr">
         <is>
-          <t>VPP2 2021716ADM.</t>
+          <t>VPP1 2004622ADM. FIDELIDAD -</t>
         </is>
       </c>
     </row>
@@ -8304,11 +8300,11 @@
       </c>
       <c r="D378" s="10" t="inlineStr">
         <is>
-          <t>VPP2 2022342ADM.</t>
+          <t>VPP2 2021716ADM.</t>
         </is>
       </c>
       <c r="E378" s="6" t="n">
-        <v>-1075965191</v>
+        <v>-2507098292</v>
       </c>
       <c r="F378" s="10" t="inlineStr">
         <is>
@@ -8321,44 +8317,44 @@
         </is>
       </c>
       <c r="H378" s="6" t="n">
-        <v>-1075965191</v>
+        <v>-2507098292</v>
       </c>
       <c r="I378" s="11" t="inlineStr">
         <is>
-          <t>VPP2 2022342ADM.</t>
+          <t>VPP2 2021716ADM.</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="C379" s="10" t="inlineStr">
         <is>
-          <t>Descuento Cliente</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D379" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>VPP2 2022342ADM.</t>
         </is>
       </c>
       <c r="E379" s="6" t="n">
-        <v>-37.26000004360685</v>
+        <v>-1075965191</v>
       </c>
       <c r="F379" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>FACT PROVEED</t>
         </is>
       </c>
       <c r="G379" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H379" s="6" t="n">
-        <v>-37.26000004360685</v>
+        <v>-1075965191</v>
       </c>
       <c r="I379" s="11" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>VPP2 2022342ADM.</t>
         </is>
       </c>
     </row>
@@ -8370,15 +8366,15 @@
       </c>
       <c r="D380" s="10" t="inlineStr">
         <is>
-          <t>PMP1286054</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E380" s="6" t="n">
-        <v>-864163</v>
+        <v>-37.26000004360685</v>
       </c>
       <c r="F380" s="10" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G380" s="10" t="inlineStr">
@@ -8387,11 +8383,11 @@
         </is>
       </c>
       <c r="H380" s="6" t="n">
-        <v>-864163</v>
+        <v>-37.26000004360685</v>
       </c>
       <c r="I380" s="11" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado PMP1286054</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
@@ -8403,11 +8399,11 @@
       </c>
       <c r="D381" s="10" t="inlineStr">
         <is>
-          <t>PMP1286550</t>
+          <t>PMP1286054</t>
         </is>
       </c>
       <c r="E381" s="6" t="n">
-        <v>-5910046.859999999</v>
+        <v>-864163</v>
       </c>
       <c r="F381" s="10" t="inlineStr">
         <is>
@@ -8420,11 +8416,11 @@
         </is>
       </c>
       <c r="H381" s="6" t="n">
-        <v>-5910046.859999999</v>
+        <v>-864163</v>
       </c>
       <c r="I381" s="11" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado PMP1286550</t>
+          <t>Menor Vlr Pagado PMP1286054</t>
         </is>
       </c>
     </row>
@@ -8436,61 +8432,61 @@
       </c>
       <c r="D382" s="10" t="inlineStr">
         <is>
-          <t>PMP1286553</t>
+          <t>PMP1286550</t>
         </is>
       </c>
       <c r="E382" s="6" t="n">
-        <v>5910047.02</v>
+        <v>-5910046.859999999</v>
       </c>
       <c r="F382" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>Menor Vlr Pagado</t>
         </is>
       </c>
       <c r="G382" s="10" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H382" s="6" t="n">
-        <v>5910047.02</v>
+        <v>-5910046.859999999</v>
       </c>
       <c r="I382" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1286553</t>
+          <t>Menor Vlr Pagado PMP1286550</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="C383" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D383" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO APERTURA</t>
+          <t>PMP1286553</t>
         </is>
       </c>
       <c r="E383" s="6" t="n">
-        <v>-14258141</v>
+        <v>5910047.02</v>
       </c>
       <c r="F383" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Myr Vlr Pagado</t>
         </is>
       </c>
       <c r="G383" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>388</t>
         </is>
       </c>
       <c r="H383" s="6" t="n">
-        <v>-14258141</v>
+        <v>5910047.02</v>
       </c>
       <c r="I383" s="11" t="inlineStr">
         <is>
-          <t>DAV DSCTO  DESCUENTO APERTURA PERFUME</t>
+          <t>Myr Vlr Pagado PMP1286553</t>
         </is>
       </c>
     </row>
@@ -8502,11 +8498,11 @@
       </c>
       <c r="D384" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>DESCUENTO APERTURA</t>
         </is>
       </c>
       <c r="E384" s="6" t="n">
-        <v>-1758901158</v>
+        <v>-14258141</v>
       </c>
       <c r="F384" s="10" t="inlineStr">
         <is>
@@ -8519,11 +8515,11 @@
         </is>
       </c>
       <c r="H384" s="6" t="n">
-        <v>-1758901158</v>
+        <v>-14258141</v>
       </c>
       <c r="I384" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO  DESCUENTO CALENDARI PERFUME</t>
+          <t>DAV DSCTO  DESCUENTO APERTURA PERFUME</t>
         </is>
       </c>
     </row>
@@ -8535,11 +8531,11 @@
       </c>
       <c r="D385" s="10" t="inlineStr">
         <is>
-          <t>DEVOLUCIONES</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E385" s="6" t="n">
-        <v>-2074733</v>
+        <v>-1758901158</v>
       </c>
       <c r="F385" s="10" t="inlineStr">
         <is>
@@ -8552,11 +8548,11 @@
         </is>
       </c>
       <c r="H385" s="6" t="n">
-        <v>-2074733</v>
+        <v>-1758901158</v>
       </c>
       <c r="I385" s="11" t="inlineStr">
         <is>
-          <t>DND DSCTO  DEVOLUCIONES PERFUME</t>
+          <t>DCA DSCTO  DESCUENTO CALENDARI PERFUME</t>
         </is>
       </c>
     </row>
@@ -8568,11 +8564,11 @@
       </c>
       <c r="D386" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>DEVOLUCIONES</t>
         </is>
       </c>
       <c r="E386" s="6" t="n">
-        <v>-76656631</v>
+        <v>-2074733</v>
       </c>
       <c r="F386" s="10" t="inlineStr">
         <is>
@@ -8585,11 +8581,11 @@
         </is>
       </c>
       <c r="H386" s="6" t="n">
-        <v>-76656631</v>
+        <v>-2074733</v>
       </c>
       <c r="I386" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO  DSTO COMERCIAL FIJO PERFUME</t>
+          <t>DND DSCTO  DEVOLUCIONES PERFUME</t>
         </is>
       </c>
     </row>
@@ -8601,11 +8597,11 @@
       </c>
       <c r="D387" s="10" t="inlineStr">
         <is>
-          <t>DTO POR ESCALA VOLU</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E387" s="6" t="n">
-        <v>-165350199</v>
+        <v>-76656631</v>
       </c>
       <c r="F387" s="10" t="inlineStr">
         <is>
@@ -8618,11 +8614,11 @@
         </is>
       </c>
       <c r="H387" s="6" t="n">
-        <v>-165350199</v>
+        <v>-76656631</v>
       </c>
       <c r="I387" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO  DTO POR ESCALA VOLU PERFUME</t>
+          <t>DCF DSCTO  DSTO COMERCIAL FIJO PERFUME</t>
         </is>
       </c>
     </row>
@@ -8638,7 +8634,7 @@
         </is>
       </c>
       <c r="E388" s="6" t="n">
-        <v>-1792140</v>
+        <v>-165350199</v>
       </c>
       <c r="F388" s="10" t="inlineStr">
         <is>
@@ -8651,11 +8647,11 @@
         </is>
       </c>
       <c r="H388" s="6" t="n">
-        <v>-1792140</v>
+        <v>-165350199</v>
       </c>
       <c r="I388" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20251200199299 DTO POR ESCALA VOLU PERFUME</t>
+          <t>DEC DSCTO  DTO POR ESCALA VOLU PERFUME</t>
         </is>
       </c>
     </row>
@@ -8671,7 +8667,7 @@
         </is>
       </c>
       <c r="E389" s="6" t="n">
-        <v>-1379112</v>
+        <v>-1792140</v>
       </c>
       <c r="F389" s="10" t="inlineStr">
         <is>
@@ -8684,11 +8680,11 @@
         </is>
       </c>
       <c r="H389" s="6" t="n">
-        <v>-1379112</v>
+        <v>-1792140</v>
       </c>
       <c r="I389" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20251200199300 DTO POR ESCALA VOLU PERFUME</t>
+          <t>DEC DSCTO 20251200199299 DTO POR ESCALA VOLU PERFUME</t>
         </is>
       </c>
     </row>
@@ -8704,7 +8700,7 @@
         </is>
       </c>
       <c r="E390" s="6" t="n">
-        <v>-80813</v>
+        <v>-1379112</v>
       </c>
       <c r="F390" s="10" t="inlineStr">
         <is>
@@ -8717,11 +8713,11 @@
         </is>
       </c>
       <c r="H390" s="6" t="n">
-        <v>-80813</v>
+        <v>-1379112</v>
       </c>
       <c r="I390" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20251200199301 DTO POR ESCALA VOLU PERFUME</t>
+          <t>DEC DSCTO 20251200199300 DTO POR ESCALA VOLU PERFUME</t>
         </is>
       </c>
     </row>
@@ -8737,7 +8733,7 @@
         </is>
       </c>
       <c r="E391" s="6" t="n">
-        <v>-470000</v>
+        <v>-80813</v>
       </c>
       <c r="F391" s="10" t="inlineStr">
         <is>
@@ -8750,11 +8746,11 @@
         </is>
       </c>
       <c r="H391" s="6" t="n">
-        <v>-470000</v>
+        <v>-80813</v>
       </c>
       <c r="I391" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20251200200041 DTO POR ESCALA VOLU PERFUME</t>
+          <t>DEC DSCTO 20251200199301 DTO POR ESCALA VOLU PERFUME</t>
         </is>
       </c>
     </row>
@@ -8766,15 +8762,15 @@
       </c>
       <c r="D392" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>DTO POR ESCALA VOLU</t>
         </is>
       </c>
       <c r="E392" s="6" t="n">
-        <v>-13427534</v>
+        <v>-470000</v>
       </c>
       <c r="F392" s="10" t="inlineStr">
         <is>
-          <t>PLATOS</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G392" s="10" t="inlineStr">
@@ -8783,11 +8779,11 @@
         </is>
       </c>
       <c r="H392" s="6" t="n">
-        <v>-13427534</v>
+        <v>-470000</v>
       </c>
       <c r="I392" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO  DESCUENTO CALENDARI PLATOS</t>
+          <t>DEC DSCTO 20251200200041 DTO POR ESCALA VOLU PERFUME</t>
         </is>
       </c>
     </row>
@@ -8799,11 +8795,11 @@
       </c>
       <c r="D393" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO COMPRAS</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E393" s="6" t="n">
-        <v>-1394767</v>
+        <v>-13427534</v>
       </c>
       <c r="F393" s="10" t="inlineStr">
         <is>
@@ -8816,11 +8812,11 @@
         </is>
       </c>
       <c r="H393" s="6" t="n">
-        <v>-1394767</v>
+        <v>-13427534</v>
       </c>
       <c r="I393" s="11" t="inlineStr">
         <is>
-          <t>DCC DSCTO  DESCUENTO COMPRAS PLATOS</t>
+          <t>DCA DSCTO  DESCUENTO CALENDARI PLATOS</t>
         </is>
       </c>
     </row>
@@ -8832,11 +8828,11 @@
       </c>
       <c r="D394" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>DESCUENTO COMPRAS</t>
         </is>
       </c>
       <c r="E394" s="6" t="n">
-        <v>-20921503</v>
+        <v>-1394767</v>
       </c>
       <c r="F394" s="10" t="inlineStr">
         <is>
@@ -8849,11 +8845,11 @@
         </is>
       </c>
       <c r="H394" s="6" t="n">
-        <v>-20921503</v>
+        <v>-1394767</v>
       </c>
       <c r="I394" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO  DSTO COMERCIAL FIJO PLATOS</t>
+          <t>DCC DSCTO  DESCUENTO COMPRAS PLATOS</t>
         </is>
       </c>
     </row>
@@ -8865,15 +8861,15 @@
       </c>
       <c r="D395" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E395" s="6" t="n">
-        <v>-61299192</v>
+        <v>-20921503</v>
       </c>
       <c r="F395" s="10" t="inlineStr">
         <is>
-          <t>RANCHO</t>
+          <t>PLATOS</t>
         </is>
       </c>
       <c r="G395" s="10" t="inlineStr">
@@ -8882,11 +8878,11 @@
         </is>
       </c>
       <c r="H395" s="6" t="n">
-        <v>-61299192</v>
+        <v>-20921503</v>
       </c>
       <c r="I395" s="11" t="inlineStr">
         <is>
-          <t>RPL DSCTO  DESCUENTO RANCHO</t>
+          <t>DCF DSCTO  DSTO COMERCIAL FIJO PLATOS</t>
         </is>
       </c>
     </row>
@@ -8898,11 +8894,11 @@
       </c>
       <c r="D396" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>DESCUENTO</t>
         </is>
       </c>
       <c r="E396" s="6" t="n">
-        <v>-29638456</v>
+        <v>-61299192</v>
       </c>
       <c r="F396" s="10" t="inlineStr">
         <is>
@@ -8915,11 +8911,11 @@
         </is>
       </c>
       <c r="H396" s="6" t="n">
-        <v>-29638456</v>
+        <v>-61299192</v>
       </c>
       <c r="I396" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO  DESCUENTO CALENDARI RANCHO</t>
+          <t>RPL DSCTO  DESCUENTO RANCHO</t>
         </is>
       </c>
     </row>
@@ -8931,11 +8927,11 @@
       </c>
       <c r="D397" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO EN PRIMER</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E397" s="6" t="n">
-        <v>-10216531</v>
+        <v>-29638456</v>
       </c>
       <c r="F397" s="10" t="inlineStr">
         <is>
@@ -8948,11 +8944,11 @@
         </is>
       </c>
       <c r="H397" s="6" t="n">
-        <v>-10216531</v>
+        <v>-29638456</v>
       </c>
       <c r="I397" s="11" t="inlineStr">
         <is>
-          <t>DPC DSCTO  DESCUENTO EN PRIMER RANCHO</t>
+          <t>DCA DSCTO  DESCUENTO CALENDARI RANCHO</t>
         </is>
       </c>
     </row>
@@ -8964,28 +8960,28 @@
       </c>
       <c r="D398" s="10" t="inlineStr">
         <is>
-          <t>PMP1282099</t>
+          <t>DESCUENTO EN PRIMER</t>
         </is>
       </c>
       <c r="E398" s="6" t="n">
-        <v>-307519</v>
+        <v>-10216531</v>
       </c>
       <c r="F398" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>RANCHO</t>
         </is>
       </c>
       <c r="G398" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H398" s="6" t="n">
-        <v>-307519</v>
+        <v>-10216531</v>
       </c>
       <c r="I398" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1282099</t>
+          <t>DPC DSCTO  DESCUENTO EN PRIMER RANCHO</t>
         </is>
       </c>
     </row>
@@ -8997,11 +8993,11 @@
       </c>
       <c r="D399" s="10" t="inlineStr">
         <is>
-          <t>PMP1282353</t>
+          <t>PMP1282099</t>
         </is>
       </c>
       <c r="E399" s="6" t="n">
-        <v>-2659670</v>
+        <v>-307519</v>
       </c>
       <c r="F399" s="10" t="inlineStr">
         <is>
@@ -9014,11 +9010,11 @@
         </is>
       </c>
       <c r="H399" s="6" t="n">
-        <v>-2659670</v>
+        <v>-307519</v>
       </c>
       <c r="I399" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1282353</t>
+          <t>Rechazo PMP1282099</t>
         </is>
       </c>
     </row>
@@ -9030,11 +9026,11 @@
       </c>
       <c r="D400" s="10" t="inlineStr">
         <is>
-          <t>PMP1282964</t>
+          <t>PMP1282353</t>
         </is>
       </c>
       <c r="E400" s="6" t="n">
-        <v>-185365</v>
+        <v>-2659670</v>
       </c>
       <c r="F400" s="10" t="inlineStr">
         <is>
@@ -9047,11 +9043,11 @@
         </is>
       </c>
       <c r="H400" s="6" t="n">
-        <v>-185365</v>
+        <v>-2659670</v>
       </c>
       <c r="I400" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1282964</t>
+          <t>Rechazo PMP1282353</t>
         </is>
       </c>
     </row>
@@ -9063,11 +9059,11 @@
       </c>
       <c r="D401" s="10" t="inlineStr">
         <is>
-          <t>PMP1283008</t>
+          <t>PMP1282964</t>
         </is>
       </c>
       <c r="E401" s="6" t="n">
-        <v>-9788</v>
+        <v>-185365</v>
       </c>
       <c r="F401" s="10" t="inlineStr">
         <is>
@@ -9080,11 +9076,11 @@
         </is>
       </c>
       <c r="H401" s="6" t="n">
-        <v>-9788</v>
+        <v>-185365</v>
       </c>
       <c r="I401" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283008</t>
+          <t>Rechazo PMP1282964</t>
         </is>
       </c>
     </row>
@@ -9096,11 +9092,11 @@
       </c>
       <c r="D402" s="10" t="inlineStr">
         <is>
-          <t>PMP1283012</t>
+          <t>PMP1283008</t>
         </is>
       </c>
       <c r="E402" s="6" t="n">
-        <v>-167913</v>
+        <v>-9788</v>
       </c>
       <c r="F402" s="10" t="inlineStr">
         <is>
@@ -9113,11 +9109,11 @@
         </is>
       </c>
       <c r="H402" s="6" t="n">
-        <v>-167913</v>
+        <v>-9788</v>
       </c>
       <c r="I402" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283012</t>
+          <t>Rechazo PMP1283008</t>
         </is>
       </c>
     </row>
@@ -9129,11 +9125,11 @@
       </c>
       <c r="D403" s="10" t="inlineStr">
         <is>
-          <t>PMP1283476</t>
+          <t>PMP1283012</t>
         </is>
       </c>
       <c r="E403" s="6" t="n">
-        <v>-836339</v>
+        <v>-167913</v>
       </c>
       <c r="F403" s="10" t="inlineStr">
         <is>
@@ -9146,11 +9142,11 @@
         </is>
       </c>
       <c r="H403" s="6" t="n">
-        <v>-836339</v>
+        <v>-167913</v>
       </c>
       <c r="I403" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283476</t>
+          <t>Rechazo PMP1283012</t>
         </is>
       </c>
     </row>
@@ -9162,11 +9158,11 @@
       </c>
       <c r="D404" s="10" t="inlineStr">
         <is>
-          <t>PMP1283500</t>
+          <t>PMP1283476</t>
         </is>
       </c>
       <c r="E404" s="6" t="n">
-        <v>-473742856</v>
+        <v>-836339</v>
       </c>
       <c r="F404" s="10" t="inlineStr">
         <is>
@@ -9179,11 +9175,11 @@
         </is>
       </c>
       <c r="H404" s="6" t="n">
-        <v>-473742856</v>
+        <v>-836339</v>
       </c>
       <c r="I404" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283500</t>
+          <t>Rechazo PMP1283476</t>
         </is>
       </c>
     </row>
@@ -9195,11 +9191,11 @@
       </c>
       <c r="D405" s="10" t="inlineStr">
         <is>
-          <t>PMP1283784</t>
+          <t>PMP1283500</t>
         </is>
       </c>
       <c r="E405" s="6" t="n">
-        <v>-629893</v>
+        <v>-473742856</v>
       </c>
       <c r="F405" s="10" t="inlineStr">
         <is>
@@ -9212,11 +9208,11 @@
         </is>
       </c>
       <c r="H405" s="6" t="n">
-        <v>-629893</v>
+        <v>-473742856</v>
       </c>
       <c r="I405" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283784</t>
+          <t>Rechazo PMP1283500</t>
         </is>
       </c>
     </row>
@@ -9228,11 +9224,11 @@
       </c>
       <c r="D406" s="10" t="inlineStr">
         <is>
-          <t>PMP1283785</t>
+          <t>PMP1283784</t>
         </is>
       </c>
       <c r="E406" s="6" t="n">
-        <v>-160273</v>
+        <v>-629893</v>
       </c>
       <c r="F406" s="10" t="inlineStr">
         <is>
@@ -9245,11 +9241,11 @@
         </is>
       </c>
       <c r="H406" s="6" t="n">
-        <v>-160273</v>
+        <v>-629893</v>
       </c>
       <c r="I406" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283785</t>
+          <t>Rechazo PMP1283784</t>
         </is>
       </c>
     </row>
@@ -9261,11 +9257,11 @@
       </c>
       <c r="D407" s="10" t="inlineStr">
         <is>
-          <t>PMP1284114</t>
+          <t>PMP1283785</t>
         </is>
       </c>
       <c r="E407" s="6" t="n">
-        <v>-764103</v>
+        <v>-160273</v>
       </c>
       <c r="F407" s="10" t="inlineStr">
         <is>
@@ -9278,11 +9274,11 @@
         </is>
       </c>
       <c r="H407" s="6" t="n">
-        <v>-764103</v>
+        <v>-160273</v>
       </c>
       <c r="I407" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284114</t>
+          <t>Rechazo PMP1283785</t>
         </is>
       </c>
     </row>
@@ -9294,11 +9290,11 @@
       </c>
       <c r="D408" s="10" t="inlineStr">
         <is>
-          <t>PMP1284117</t>
+          <t>PMP1284114</t>
         </is>
       </c>
       <c r="E408" s="6" t="n">
-        <v>-177051</v>
+        <v>-764103</v>
       </c>
       <c r="F408" s="10" t="inlineStr">
         <is>
@@ -9311,11 +9307,11 @@
         </is>
       </c>
       <c r="H408" s="6" t="n">
-        <v>-177051</v>
+        <v>-764103</v>
       </c>
       <c r="I408" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284117</t>
+          <t>Rechazo PMP1284114</t>
         </is>
       </c>
     </row>
@@ -9327,11 +9323,11 @@
       </c>
       <c r="D409" s="10" t="inlineStr">
         <is>
-          <t>PMP1284119</t>
+          <t>PMP1284117</t>
         </is>
       </c>
       <c r="E409" s="6" t="n">
-        <v>-644997</v>
+        <v>-177051</v>
       </c>
       <c r="F409" s="10" t="inlineStr">
         <is>
@@ -9344,11 +9340,11 @@
         </is>
       </c>
       <c r="H409" s="6" t="n">
-        <v>-644997</v>
+        <v>-177051</v>
       </c>
       <c r="I409" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284119</t>
+          <t>Rechazo PMP1284117</t>
         </is>
       </c>
     </row>
@@ -9360,11 +9356,11 @@
       </c>
       <c r="D410" s="10" t="inlineStr">
         <is>
-          <t>PMP1284200</t>
+          <t>PMP1284119</t>
         </is>
       </c>
       <c r="E410" s="6" t="n">
-        <v>-175153</v>
+        <v>-644997</v>
       </c>
       <c r="F410" s="10" t="inlineStr">
         <is>
@@ -9377,11 +9373,11 @@
         </is>
       </c>
       <c r="H410" s="6" t="n">
-        <v>-175153</v>
+        <v>-644997</v>
       </c>
       <c r="I410" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284200</t>
+          <t>Rechazo PMP1284119</t>
         </is>
       </c>
     </row>
@@ -9393,11 +9389,11 @@
       </c>
       <c r="D411" s="10" t="inlineStr">
         <is>
-          <t>PMP1284460</t>
+          <t>PMP1284200</t>
         </is>
       </c>
       <c r="E411" s="6" t="n">
-        <v>-167879</v>
+        <v>-175153</v>
       </c>
       <c r="F411" s="10" t="inlineStr">
         <is>
@@ -9410,11 +9406,11 @@
         </is>
       </c>
       <c r="H411" s="6" t="n">
-        <v>-167879</v>
+        <v>-175153</v>
       </c>
       <c r="I411" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284460</t>
+          <t>Rechazo PMP1284200</t>
         </is>
       </c>
     </row>
@@ -9426,11 +9422,11 @@
       </c>
       <c r="D412" s="10" t="inlineStr">
         <is>
-          <t>PMP1284462</t>
+          <t>PMP1284460</t>
         </is>
       </c>
       <c r="E412" s="6" t="n">
-        <v>-322931</v>
+        <v>-167879</v>
       </c>
       <c r="F412" s="10" t="inlineStr">
         <is>
@@ -9443,11 +9439,11 @@
         </is>
       </c>
       <c r="H412" s="6" t="n">
-        <v>-322931</v>
+        <v>-167879</v>
       </c>
       <c r="I412" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284462</t>
+          <t>Rechazo PMP1284460</t>
         </is>
       </c>
     </row>
@@ -9459,11 +9455,11 @@
       </c>
       <c r="D413" s="10" t="inlineStr">
         <is>
-          <t>PMP1284529</t>
+          <t>PMP1284462</t>
         </is>
       </c>
       <c r="E413" s="6" t="n">
-        <v>-276742</v>
+        <v>-322931</v>
       </c>
       <c r="F413" s="10" t="inlineStr">
         <is>
@@ -9476,11 +9472,11 @@
         </is>
       </c>
       <c r="H413" s="6" t="n">
-        <v>-276742</v>
+        <v>-322931</v>
       </c>
       <c r="I413" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284529</t>
+          <t>Rechazo PMP1284462</t>
         </is>
       </c>
     </row>
@@ -9492,11 +9488,11 @@
       </c>
       <c r="D414" s="10" t="inlineStr">
         <is>
-          <t>PMP1284543</t>
+          <t>PMP1284529</t>
         </is>
       </c>
       <c r="E414" s="6" t="n">
-        <v>-3015665</v>
+        <v>-276742</v>
       </c>
       <c r="F414" s="10" t="inlineStr">
         <is>
@@ -9509,11 +9505,11 @@
         </is>
       </c>
       <c r="H414" s="6" t="n">
-        <v>-3015665</v>
+        <v>-276742</v>
       </c>
       <c r="I414" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284543</t>
+          <t>Rechazo PMP1284529</t>
         </is>
       </c>
     </row>
@@ -9525,11 +9521,11 @@
       </c>
       <c r="D415" s="10" t="inlineStr">
         <is>
-          <t>PMP1284546</t>
+          <t>PMP1284543</t>
         </is>
       </c>
       <c r="E415" s="6" t="n">
-        <v>-135409</v>
+        <v>-3015665</v>
       </c>
       <c r="F415" s="10" t="inlineStr">
         <is>
@@ -9542,11 +9538,11 @@
         </is>
       </c>
       <c r="H415" s="6" t="n">
-        <v>-135409</v>
+        <v>-3015665</v>
       </c>
       <c r="I415" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284546</t>
+          <t>Rechazo PMP1284543</t>
         </is>
       </c>
     </row>
@@ -9558,11 +9554,11 @@
       </c>
       <c r="D416" s="10" t="inlineStr">
         <is>
-          <t>PMP1284602</t>
+          <t>PMP1284546</t>
         </is>
       </c>
       <c r="E416" s="6" t="n">
-        <v>-930108</v>
+        <v>-135409</v>
       </c>
       <c r="F416" s="10" t="inlineStr">
         <is>
@@ -9575,11 +9571,11 @@
         </is>
       </c>
       <c r="H416" s="6" t="n">
-        <v>-930108</v>
+        <v>-135409</v>
       </c>
       <c r="I416" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284602</t>
+          <t>Rechazo PMP1284546</t>
         </is>
       </c>
     </row>
@@ -9591,11 +9587,11 @@
       </c>
       <c r="D417" s="10" t="inlineStr">
         <is>
-          <t>PMP1284750</t>
+          <t>PMP1284602</t>
         </is>
       </c>
       <c r="E417" s="6" t="n">
-        <v>-405708</v>
+        <v>-930108</v>
       </c>
       <c r="F417" s="10" t="inlineStr">
         <is>
@@ -9608,11 +9604,11 @@
         </is>
       </c>
       <c r="H417" s="6" t="n">
-        <v>-405708</v>
+        <v>-930108</v>
       </c>
       <c r="I417" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284750</t>
+          <t>Rechazo PMP1284602</t>
         </is>
       </c>
     </row>
@@ -9624,11 +9620,11 @@
       </c>
       <c r="D418" s="10" t="inlineStr">
         <is>
-          <t>PMP1284800</t>
+          <t>PMP1284750</t>
         </is>
       </c>
       <c r="E418" s="6" t="n">
-        <v>-635980</v>
+        <v>-405708</v>
       </c>
       <c r="F418" s="10" t="inlineStr">
         <is>
@@ -9641,11 +9637,11 @@
         </is>
       </c>
       <c r="H418" s="6" t="n">
-        <v>-635980</v>
+        <v>-405708</v>
       </c>
       <c r="I418" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284800</t>
+          <t>Rechazo PMP1284750</t>
         </is>
       </c>
     </row>
@@ -9657,11 +9653,11 @@
       </c>
       <c r="D419" s="10" t="inlineStr">
         <is>
-          <t>PMP1284876</t>
+          <t>PMP1284800</t>
         </is>
       </c>
       <c r="E419" s="6" t="n">
-        <v>-689804</v>
+        <v>-635980</v>
       </c>
       <c r="F419" s="10" t="inlineStr">
         <is>
@@ -9674,11 +9670,11 @@
         </is>
       </c>
       <c r="H419" s="6" t="n">
-        <v>-689804</v>
+        <v>-635980</v>
       </c>
       <c r="I419" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284876</t>
+          <t>Rechazo PMP1284800</t>
         </is>
       </c>
     </row>
@@ -9690,11 +9686,11 @@
       </c>
       <c r="D420" s="10" t="inlineStr">
         <is>
-          <t>PMP1284878</t>
+          <t>PMP1284876</t>
         </is>
       </c>
       <c r="E420" s="6" t="n">
-        <v>-135533</v>
+        <v>-689804</v>
       </c>
       <c r="F420" s="10" t="inlineStr">
         <is>
@@ -9707,11 +9703,11 @@
         </is>
       </c>
       <c r="H420" s="6" t="n">
-        <v>-135533</v>
+        <v>-689804</v>
       </c>
       <c r="I420" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284878</t>
+          <t>Rechazo PMP1284876</t>
         </is>
       </c>
     </row>
@@ -9723,11 +9719,11 @@
       </c>
       <c r="D421" s="10" t="inlineStr">
         <is>
-          <t>PMP1284879</t>
+          <t>PMP1284878</t>
         </is>
       </c>
       <c r="E421" s="6" t="n">
-        <v>-732728</v>
+        <v>-135533</v>
       </c>
       <c r="F421" s="10" t="inlineStr">
         <is>
@@ -9740,11 +9736,11 @@
         </is>
       </c>
       <c r="H421" s="6" t="n">
-        <v>-732728</v>
+        <v>-135533</v>
       </c>
       <c r="I421" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284879</t>
+          <t>Rechazo PMP1284878</t>
         </is>
       </c>
     </row>
@@ -9756,11 +9752,11 @@
       </c>
       <c r="D422" s="10" t="inlineStr">
         <is>
-          <t>PMP1284948</t>
+          <t>PMP1284879</t>
         </is>
       </c>
       <c r="E422" s="6" t="n">
-        <v>-1060968</v>
+        <v>-732728</v>
       </c>
       <c r="F422" s="10" t="inlineStr">
         <is>
@@ -9773,11 +9769,11 @@
         </is>
       </c>
       <c r="H422" s="6" t="n">
-        <v>-1060968</v>
+        <v>-732728</v>
       </c>
       <c r="I422" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284948</t>
+          <t>Rechazo PMP1284879</t>
         </is>
       </c>
     </row>
@@ -9789,11 +9785,11 @@
       </c>
       <c r="D423" s="10" t="inlineStr">
         <is>
-          <t>PMP1284949</t>
+          <t>PMP1284948</t>
         </is>
       </c>
       <c r="E423" s="6" t="n">
-        <v>-215248</v>
+        <v>-1060968</v>
       </c>
       <c r="F423" s="10" t="inlineStr">
         <is>
@@ -9806,11 +9802,11 @@
         </is>
       </c>
       <c r="H423" s="6" t="n">
-        <v>-215248</v>
+        <v>-1060968</v>
       </c>
       <c r="I423" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284949</t>
+          <t>Rechazo PMP1284948</t>
         </is>
       </c>
     </row>
@@ -9822,11 +9818,11 @@
       </c>
       <c r="D424" s="10" t="inlineStr">
         <is>
-          <t>PMP1284950</t>
+          <t>PMP1284949</t>
         </is>
       </c>
       <c r="E424" s="6" t="n">
-        <v>-1297475</v>
+        <v>-215248</v>
       </c>
       <c r="F424" s="10" t="inlineStr">
         <is>
@@ -9839,11 +9835,11 @@
         </is>
       </c>
       <c r="H424" s="6" t="n">
-        <v>-1297475</v>
+        <v>-215248</v>
       </c>
       <c r="I424" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284950</t>
+          <t>Rechazo PMP1284949</t>
         </is>
       </c>
     </row>
@@ -9855,11 +9851,11 @@
       </c>
       <c r="D425" s="10" t="inlineStr">
         <is>
-          <t>PMP1284951</t>
+          <t>PMP1284950</t>
         </is>
       </c>
       <c r="E425" s="6" t="n">
-        <v>-5702098</v>
+        <v>-1297475</v>
       </c>
       <c r="F425" s="10" t="inlineStr">
         <is>
@@ -9872,11 +9868,11 @@
         </is>
       </c>
       <c r="H425" s="6" t="n">
-        <v>-5702098</v>
+        <v>-1297475</v>
       </c>
       <c r="I425" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284951</t>
+          <t>Rechazo PMP1284950</t>
         </is>
       </c>
     </row>
@@ -9888,11 +9884,11 @@
       </c>
       <c r="D426" s="10" t="inlineStr">
         <is>
-          <t>PMP1285048</t>
+          <t>PMP1284951</t>
         </is>
       </c>
       <c r="E426" s="6" t="n">
-        <v>-221603</v>
+        <v>-5702098</v>
       </c>
       <c r="F426" s="10" t="inlineStr">
         <is>
@@ -9905,11 +9901,11 @@
         </is>
       </c>
       <c r="H426" s="6" t="n">
-        <v>-221603</v>
+        <v>-5702098</v>
       </c>
       <c r="I426" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285048</t>
+          <t>Rechazo PMP1284951</t>
         </is>
       </c>
     </row>
@@ -9921,11 +9917,11 @@
       </c>
       <c r="D427" s="10" t="inlineStr">
         <is>
-          <t>PMP1285059</t>
+          <t>PMP1285048</t>
         </is>
       </c>
       <c r="E427" s="6" t="n">
-        <v>-160294</v>
+        <v>-221603</v>
       </c>
       <c r="F427" s="10" t="inlineStr">
         <is>
@@ -9938,11 +9934,11 @@
         </is>
       </c>
       <c r="H427" s="6" t="n">
-        <v>-160294</v>
+        <v>-221603</v>
       </c>
       <c r="I427" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285059</t>
+          <t>Rechazo PMP1285048</t>
         </is>
       </c>
     </row>
@@ -9954,11 +9950,11 @@
       </c>
       <c r="D428" s="10" t="inlineStr">
         <is>
-          <t>PMP1285065</t>
+          <t>PMP1285059</t>
         </is>
       </c>
       <c r="E428" s="6" t="n">
-        <v>-107552</v>
+        <v>-160294</v>
       </c>
       <c r="F428" s="10" t="inlineStr">
         <is>
@@ -9971,11 +9967,11 @@
         </is>
       </c>
       <c r="H428" s="6" t="n">
-        <v>-107552</v>
+        <v>-160294</v>
       </c>
       <c r="I428" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285065</t>
+          <t>Rechazo PMP1285059</t>
         </is>
       </c>
     </row>
@@ -9987,11 +9983,11 @@
       </c>
       <c r="D429" s="10" t="inlineStr">
         <is>
-          <t>PMP1285067</t>
+          <t>PMP1285065</t>
         </is>
       </c>
       <c r="E429" s="6" t="n">
-        <v>-135307</v>
+        <v>-107552</v>
       </c>
       <c r="F429" s="10" t="inlineStr">
         <is>
@@ -10004,11 +10000,11 @@
         </is>
       </c>
       <c r="H429" s="6" t="n">
-        <v>-135307</v>
+        <v>-107552</v>
       </c>
       <c r="I429" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285067</t>
+          <t>Rechazo PMP1285065</t>
         </is>
       </c>
     </row>
@@ -10020,11 +10016,11 @@
       </c>
       <c r="D430" s="10" t="inlineStr">
         <is>
-          <t>PMP1285071</t>
+          <t>PMP1285067</t>
         </is>
       </c>
       <c r="E430" s="6" t="n">
-        <v>-419436</v>
+        <v>-135307</v>
       </c>
       <c r="F430" s="10" t="inlineStr">
         <is>
@@ -10037,11 +10033,11 @@
         </is>
       </c>
       <c r="H430" s="6" t="n">
-        <v>-419436</v>
+        <v>-135307</v>
       </c>
       <c r="I430" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285071</t>
+          <t>Rechazo PMP1285067</t>
         </is>
       </c>
     </row>
@@ -10053,11 +10049,11 @@
       </c>
       <c r="D431" s="10" t="inlineStr">
         <is>
-          <t>PMP1285653</t>
+          <t>PMP1285071</t>
         </is>
       </c>
       <c r="E431" s="6" t="n">
-        <v>-558246</v>
+        <v>-419436</v>
       </c>
       <c r="F431" s="10" t="inlineStr">
         <is>
@@ -10070,11 +10066,11 @@
         </is>
       </c>
       <c r="H431" s="6" t="n">
-        <v>-558246</v>
+        <v>-419436</v>
       </c>
       <c r="I431" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285653</t>
+          <t>Rechazo PMP1285071</t>
         </is>
       </c>
     </row>
@@ -10086,11 +10082,11 @@
       </c>
       <c r="D432" s="10" t="inlineStr">
         <is>
-          <t>PMP1285659</t>
+          <t>PMP1285653</t>
         </is>
       </c>
       <c r="E432" s="6" t="n">
-        <v>-311765</v>
+        <v>-558246</v>
       </c>
       <c r="F432" s="10" t="inlineStr">
         <is>
@@ -10103,11 +10099,11 @@
         </is>
       </c>
       <c r="H432" s="6" t="n">
-        <v>-311765</v>
+        <v>-558246</v>
       </c>
       <c r="I432" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285659</t>
+          <t>Rechazo PMP1285653</t>
         </is>
       </c>
     </row>
@@ -10119,11 +10115,11 @@
       </c>
       <c r="D433" s="10" t="inlineStr">
         <is>
-          <t>PMP1285725</t>
+          <t>PMP1285659</t>
         </is>
       </c>
       <c r="E433" s="6" t="n">
-        <v>-679290</v>
+        <v>-311765</v>
       </c>
       <c r="F433" s="10" t="inlineStr">
         <is>
@@ -10136,11 +10132,11 @@
         </is>
       </c>
       <c r="H433" s="6" t="n">
-        <v>-679290</v>
+        <v>-311765</v>
       </c>
       <c r="I433" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285725</t>
+          <t>Rechazo PMP1285659</t>
         </is>
       </c>
     </row>
@@ -10152,11 +10148,11 @@
       </c>
       <c r="D434" s="10" t="inlineStr">
         <is>
-          <t>PMP1285898</t>
+          <t>PMP1285725</t>
         </is>
       </c>
       <c r="E434" s="6" t="n">
-        <v>-253685</v>
+        <v>-679290</v>
       </c>
       <c r="F434" s="10" t="inlineStr">
         <is>
@@ -10169,11 +10165,11 @@
         </is>
       </c>
       <c r="H434" s="6" t="n">
-        <v>-253685</v>
+        <v>-679290</v>
       </c>
       <c r="I434" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285898</t>
+          <t>Rechazo PMP1285725</t>
         </is>
       </c>
     </row>
@@ -10185,11 +10181,11 @@
       </c>
       <c r="D435" s="10" t="inlineStr">
         <is>
-          <t>PMP1285903</t>
+          <t>PMP1285898</t>
         </is>
       </c>
       <c r="E435" s="6" t="n">
-        <v>-322554</v>
+        <v>-253685</v>
       </c>
       <c r="F435" s="10" t="inlineStr">
         <is>
@@ -10202,11 +10198,11 @@
         </is>
       </c>
       <c r="H435" s="6" t="n">
-        <v>-322554</v>
+        <v>-253685</v>
       </c>
       <c r="I435" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285903</t>
+          <t>Rechazo PMP1285898</t>
         </is>
       </c>
     </row>
@@ -10218,11 +10214,11 @@
       </c>
       <c r="D436" s="10" t="inlineStr">
         <is>
-          <t>PMP1285908</t>
+          <t>PMP1285903</t>
         </is>
       </c>
       <c r="E436" s="6" t="n">
-        <v>-135255</v>
+        <v>-322554</v>
       </c>
       <c r="F436" s="10" t="inlineStr">
         <is>
@@ -10235,11 +10231,11 @@
         </is>
       </c>
       <c r="H436" s="6" t="n">
-        <v>-135255</v>
+        <v>-322554</v>
       </c>
       <c r="I436" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285908</t>
+          <t>Rechazo PMP1285903</t>
         </is>
       </c>
     </row>
@@ -10251,11 +10247,11 @@
       </c>
       <c r="D437" s="10" t="inlineStr">
         <is>
-          <t>PMP1286056</t>
+          <t>PMP1285908</t>
         </is>
       </c>
       <c r="E437" s="6" t="n">
-        <v>-556413</v>
+        <v>-135255</v>
       </c>
       <c r="F437" s="10" t="inlineStr">
         <is>
@@ -10268,11 +10264,11 @@
         </is>
       </c>
       <c r="H437" s="6" t="n">
-        <v>-556413</v>
+        <v>-135255</v>
       </c>
       <c r="I437" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286056</t>
+          <t>Rechazo PMP1285908</t>
         </is>
       </c>
     </row>
@@ -10284,11 +10280,11 @@
       </c>
       <c r="D438" s="10" t="inlineStr">
         <is>
-          <t>PMP1286208</t>
+          <t>PMP1286056</t>
         </is>
       </c>
       <c r="E438" s="6" t="n">
-        <v>-949123</v>
+        <v>-556413</v>
       </c>
       <c r="F438" s="10" t="inlineStr">
         <is>
@@ -10301,11 +10297,11 @@
         </is>
       </c>
       <c r="H438" s="6" t="n">
-        <v>-949123</v>
+        <v>-556413</v>
       </c>
       <c r="I438" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286208</t>
+          <t>Rechazo PMP1286056</t>
         </is>
       </c>
     </row>
@@ -10317,11 +10313,11 @@
       </c>
       <c r="D439" s="10" t="inlineStr">
         <is>
-          <t>PMP1286554</t>
+          <t>PMP1286208</t>
         </is>
       </c>
       <c r="E439" s="6" t="n">
-        <v>-354934</v>
+        <v>-949123</v>
       </c>
       <c r="F439" s="10" t="inlineStr">
         <is>
@@ -10334,11 +10330,11 @@
         </is>
       </c>
       <c r="H439" s="6" t="n">
-        <v>-354934</v>
+        <v>-949123</v>
       </c>
       <c r="I439" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286554</t>
+          <t>Rechazo PMP1286208</t>
         </is>
       </c>
     </row>
@@ -10350,11 +10346,11 @@
       </c>
       <c r="D440" s="10" t="inlineStr">
         <is>
-          <t>PMP1286556</t>
+          <t>PMP1286554</t>
         </is>
       </c>
       <c r="E440" s="6" t="n">
-        <v>-364001</v>
+        <v>-354934</v>
       </c>
       <c r="F440" s="10" t="inlineStr">
         <is>
@@ -10367,11 +10363,11 @@
         </is>
       </c>
       <c r="H440" s="6" t="n">
-        <v>-364001</v>
+        <v>-354934</v>
       </c>
       <c r="I440" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286556</t>
+          <t>Rechazo PMP1286554</t>
         </is>
       </c>
     </row>
@@ -10383,11 +10379,11 @@
       </c>
       <c r="D441" s="10" t="inlineStr">
         <is>
-          <t>PMP1286709</t>
+          <t>PMP1286556</t>
         </is>
       </c>
       <c r="E441" s="6" t="n">
-        <v>-33537478</v>
+        <v>-364001</v>
       </c>
       <c r="F441" s="10" t="inlineStr">
         <is>
@@ -10400,11 +10396,11 @@
         </is>
       </c>
       <c r="H441" s="6" t="n">
-        <v>-33537478</v>
+        <v>-364001</v>
       </c>
       <c r="I441" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286709</t>
+          <t>Rechazo PMP1286556</t>
         </is>
       </c>
     </row>
@@ -10416,11 +10412,11 @@
       </c>
       <c r="D442" s="10" t="inlineStr">
         <is>
-          <t>PMP1286710</t>
+          <t>PMP1286709</t>
         </is>
       </c>
       <c r="E442" s="6" t="n">
-        <v>-650618</v>
+        <v>-33537478</v>
       </c>
       <c r="F442" s="10" t="inlineStr">
         <is>
@@ -10433,11 +10429,11 @@
         </is>
       </c>
       <c r="H442" s="6" t="n">
-        <v>-650618</v>
+        <v>-33537478</v>
       </c>
       <c r="I442" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286710</t>
+          <t>Rechazo PMP1286709</t>
         </is>
       </c>
     </row>
@@ -10449,11 +10445,11 @@
       </c>
       <c r="D443" s="10" t="inlineStr">
         <is>
-          <t>PMP1286711</t>
+          <t>PMP1286710</t>
         </is>
       </c>
       <c r="E443" s="6" t="n">
-        <v>-6920570</v>
+        <v>-650618</v>
       </c>
       <c r="F443" s="10" t="inlineStr">
         <is>
@@ -10466,11 +10462,11 @@
         </is>
       </c>
       <c r="H443" s="6" t="n">
-        <v>-6920570</v>
+        <v>-650618</v>
       </c>
       <c r="I443" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286711</t>
+          <t>Rechazo PMP1286710</t>
         </is>
       </c>
     </row>
@@ -10482,11 +10478,11 @@
       </c>
       <c r="D444" s="10" t="inlineStr">
         <is>
-          <t>PMP1286712</t>
+          <t>PMP1286711</t>
         </is>
       </c>
       <c r="E444" s="6" t="n">
-        <v>-403395</v>
+        <v>-6920570</v>
       </c>
       <c r="F444" s="10" t="inlineStr">
         <is>
@@ -10499,11 +10495,11 @@
         </is>
       </c>
       <c r="H444" s="6" t="n">
-        <v>-403395</v>
+        <v>-6920570</v>
       </c>
       <c r="I444" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286712</t>
+          <t>Rechazo PMP1286711</t>
         </is>
       </c>
     </row>
@@ -10515,11 +10511,11 @@
       </c>
       <c r="D445" s="10" t="inlineStr">
         <is>
-          <t>PMP1286715</t>
+          <t>PMP1286712</t>
         </is>
       </c>
       <c r="E445" s="6" t="n">
-        <v>-4085189</v>
+        <v>-403395</v>
       </c>
       <c r="F445" s="10" t="inlineStr">
         <is>
@@ -10532,11 +10528,11 @@
         </is>
       </c>
       <c r="H445" s="6" t="n">
-        <v>-4085189</v>
+        <v>-403395</v>
       </c>
       <c r="I445" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286715</t>
+          <t>Rechazo PMP1286712</t>
         </is>
       </c>
     </row>
@@ -10548,11 +10544,11 @@
       </c>
       <c r="D446" s="10" t="inlineStr">
         <is>
-          <t>PMP1286716</t>
+          <t>PMP1286715</t>
         </is>
       </c>
       <c r="E446" s="6" t="n">
-        <v>-822039</v>
+        <v>-4085189</v>
       </c>
       <c r="F446" s="10" t="inlineStr">
         <is>
@@ -10565,11 +10561,11 @@
         </is>
       </c>
       <c r="H446" s="6" t="n">
-        <v>-822039</v>
+        <v>-4085189</v>
       </c>
       <c r="I446" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286716</t>
+          <t>Rechazo PMP1286715</t>
         </is>
       </c>
     </row>
@@ -10581,11 +10577,11 @@
       </c>
       <c r="D447" s="10" t="inlineStr">
         <is>
-          <t>PMP1287257</t>
+          <t>PMP1286716</t>
         </is>
       </c>
       <c r="E447" s="6" t="n">
-        <v>-156625</v>
+        <v>-822039</v>
       </c>
       <c r="F447" s="10" t="inlineStr">
         <is>
@@ -10598,11 +10594,11 @@
         </is>
       </c>
       <c r="H447" s="6" t="n">
-        <v>-156625</v>
+        <v>-822039</v>
       </c>
       <c r="I447" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287257</t>
+          <t>Rechazo PMP1286716</t>
         </is>
       </c>
     </row>
@@ -10614,11 +10610,11 @@
       </c>
       <c r="D448" s="10" t="inlineStr">
         <is>
-          <t>PMP1287321</t>
+          <t>PMP1287257</t>
         </is>
       </c>
       <c r="E448" s="6" t="n">
-        <v>-182163</v>
+        <v>-156625</v>
       </c>
       <c r="F448" s="10" t="inlineStr">
         <is>
@@ -10631,11 +10627,11 @@
         </is>
       </c>
       <c r="H448" s="6" t="n">
-        <v>-182163</v>
+        <v>-156625</v>
       </c>
       <c r="I448" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287321</t>
+          <t>Rechazo PMP1287257</t>
         </is>
       </c>
     </row>
@@ -10647,11 +10643,11 @@
       </c>
       <c r="D449" s="10" t="inlineStr">
         <is>
-          <t>PMP1287325</t>
+          <t>PMP1287321</t>
         </is>
       </c>
       <c r="E449" s="6" t="n">
-        <v>-118625</v>
+        <v>-182163</v>
       </c>
       <c r="F449" s="10" t="inlineStr">
         <is>
@@ -10664,11 +10660,11 @@
         </is>
       </c>
       <c r="H449" s="6" t="n">
-        <v>-118625</v>
+        <v>-182163</v>
       </c>
       <c r="I449" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287325</t>
+          <t>Rechazo PMP1287321</t>
         </is>
       </c>
     </row>
@@ -10680,11 +10676,11 @@
       </c>
       <c r="D450" s="10" t="inlineStr">
         <is>
-          <t>PMP1287335</t>
+          <t>PMP1287325</t>
         </is>
       </c>
       <c r="E450" s="6" t="n">
-        <v>-128620</v>
+        <v>-118625</v>
       </c>
       <c r="F450" s="10" t="inlineStr">
         <is>
@@ -10697,11 +10693,11 @@
         </is>
       </c>
       <c r="H450" s="6" t="n">
-        <v>-128620</v>
+        <v>-118625</v>
       </c>
       <c r="I450" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287335</t>
+          <t>Rechazo PMP1287325</t>
         </is>
       </c>
     </row>
@@ -10713,11 +10709,11 @@
       </c>
       <c r="D451" s="10" t="inlineStr">
         <is>
-          <t>PMP1287379</t>
+          <t>PMP1287335</t>
         </is>
       </c>
       <c r="E451" s="6" t="n">
-        <v>-271757</v>
+        <v>-128620</v>
       </c>
       <c r="F451" s="10" t="inlineStr">
         <is>
@@ -10730,11 +10726,11 @@
         </is>
       </c>
       <c r="H451" s="6" t="n">
-        <v>-271757</v>
+        <v>-128620</v>
       </c>
       <c r="I451" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287379</t>
+          <t>Rechazo PMP1287335</t>
         </is>
       </c>
     </row>
@@ -10746,11 +10742,11 @@
       </c>
       <c r="D452" s="10" t="inlineStr">
         <is>
-          <t>PMP1287385</t>
+          <t>PMP1287379</t>
         </is>
       </c>
       <c r="E452" s="6" t="n">
-        <v>-214996</v>
+        <v>-271757</v>
       </c>
       <c r="F452" s="10" t="inlineStr">
         <is>
@@ -10763,11 +10759,11 @@
         </is>
       </c>
       <c r="H452" s="6" t="n">
-        <v>-214996</v>
+        <v>-271757</v>
       </c>
       <c r="I452" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287385</t>
+          <t>Rechazo PMP1287379</t>
         </is>
       </c>
     </row>
@@ -10779,11 +10775,11 @@
       </c>
       <c r="D453" s="10" t="inlineStr">
         <is>
-          <t>PMP1287386</t>
+          <t>PMP1287385</t>
         </is>
       </c>
       <c r="E453" s="6" t="n">
-        <v>-267680</v>
+        <v>-214996</v>
       </c>
       <c r="F453" s="10" t="inlineStr">
         <is>
@@ -10796,11 +10792,11 @@
         </is>
       </c>
       <c r="H453" s="6" t="n">
-        <v>-267680</v>
+        <v>-214996</v>
       </c>
       <c r="I453" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287386</t>
+          <t>Rechazo PMP1287385</t>
         </is>
       </c>
     </row>
@@ -10812,11 +10808,11 @@
       </c>
       <c r="D454" s="10" t="inlineStr">
         <is>
-          <t>PMP1287574</t>
+          <t>PMP1287386</t>
         </is>
       </c>
       <c r="E454" s="6" t="n">
-        <v>-11940004</v>
+        <v>-267680</v>
       </c>
       <c r="F454" s="10" t="inlineStr">
         <is>
@@ -10829,11 +10825,11 @@
         </is>
       </c>
       <c r="H454" s="6" t="n">
-        <v>-11940004</v>
+        <v>-267680</v>
       </c>
       <c r="I454" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287574</t>
+          <t>Rechazo PMP1287386</t>
         </is>
       </c>
     </row>
@@ -10845,11 +10841,11 @@
       </c>
       <c r="D455" s="10" t="inlineStr">
         <is>
-          <t>PMP1287736</t>
+          <t>PMP1287574</t>
         </is>
       </c>
       <c r="E455" s="6" t="n">
-        <v>-93440</v>
+        <v>-11940004</v>
       </c>
       <c r="F455" s="10" t="inlineStr">
         <is>
@@ -10862,11 +10858,11 @@
         </is>
       </c>
       <c r="H455" s="6" t="n">
-        <v>-93440</v>
+        <v>-11940004</v>
       </c>
       <c r="I455" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287736</t>
+          <t>Rechazo PMP1287574</t>
         </is>
       </c>
     </row>
@@ -10878,11 +10874,11 @@
       </c>
       <c r="D456" s="10" t="inlineStr">
         <is>
-          <t>PMP128777746</t>
+          <t>PMP1287736</t>
         </is>
       </c>
       <c r="E456" s="6" t="n">
-        <v>-322500</v>
+        <v>-93440</v>
       </c>
       <c r="F456" s="10" t="inlineStr">
         <is>
@@ -10895,11 +10891,11 @@
         </is>
       </c>
       <c r="H456" s="6" t="n">
-        <v>-322500</v>
+        <v>-93440</v>
       </c>
       <c r="I456" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP128777746</t>
+          <t>Rechazo PMP1287736</t>
         </is>
       </c>
     </row>
@@ -10911,11 +10907,11 @@
       </c>
       <c r="D457" s="10" t="inlineStr">
         <is>
-          <t>PMP1287829</t>
+          <t>PMP128777746</t>
         </is>
       </c>
       <c r="E457" s="6" t="n">
-        <v>-290823</v>
+        <v>-322500</v>
       </c>
       <c r="F457" s="10" t="inlineStr">
         <is>
@@ -10928,11 +10924,11 @@
         </is>
       </c>
       <c r="H457" s="6" t="n">
-        <v>-290823</v>
+        <v>-322500</v>
       </c>
       <c r="I457" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287829</t>
+          <t>Rechazo PMP128777746</t>
         </is>
       </c>
     </row>
@@ -10944,11 +10940,11 @@
       </c>
       <c r="D458" s="10" t="inlineStr">
         <is>
-          <t>PMP1287903</t>
+          <t>PMP1287829</t>
         </is>
       </c>
       <c r="E458" s="6" t="n">
-        <v>-128514</v>
+        <v>-290823</v>
       </c>
       <c r="F458" s="10" t="inlineStr">
         <is>
@@ -10961,11 +10957,11 @@
         </is>
       </c>
       <c r="H458" s="6" t="n">
-        <v>-128514</v>
+        <v>-290823</v>
       </c>
       <c r="I458" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287903</t>
+          <t>Rechazo PMP1287829</t>
         </is>
       </c>
     </row>
@@ -10977,11 +10973,11 @@
       </c>
       <c r="D459" s="10" t="inlineStr">
         <is>
-          <t>PMP1287904</t>
+          <t>PMP1287903</t>
         </is>
       </c>
       <c r="E459" s="6" t="n">
-        <v>-80064</v>
+        <v>-128514</v>
       </c>
       <c r="F459" s="10" t="inlineStr">
         <is>
@@ -10994,11 +10990,11 @@
         </is>
       </c>
       <c r="H459" s="6" t="n">
-        <v>-80064</v>
+        <v>-128514</v>
       </c>
       <c r="I459" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287904</t>
+          <t>Rechazo PMP1287903</t>
         </is>
       </c>
     </row>
@@ -11010,11 +11006,11 @@
       </c>
       <c r="D460" s="10" t="inlineStr">
         <is>
-          <t>PMP1287920</t>
+          <t>PMP1287904</t>
         </is>
       </c>
       <c r="E460" s="6" t="n">
-        <v>-582605</v>
+        <v>-80064</v>
       </c>
       <c r="F460" s="10" t="inlineStr">
         <is>
@@ -11027,11 +11023,11 @@
         </is>
       </c>
       <c r="H460" s="6" t="n">
-        <v>-582605</v>
+        <v>-80064</v>
       </c>
       <c r="I460" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287920</t>
+          <t>Rechazo PMP1287904</t>
         </is>
       </c>
     </row>
@@ -11043,11 +11039,11 @@
       </c>
       <c r="D461" s="10" t="inlineStr">
         <is>
-          <t>PMP1287921</t>
+          <t>PMP1287920</t>
         </is>
       </c>
       <c r="E461" s="6" t="n">
-        <v>-124374</v>
+        <v>-582605</v>
       </c>
       <c r="F461" s="10" t="inlineStr">
         <is>
@@ -11060,11 +11056,11 @@
         </is>
       </c>
       <c r="H461" s="6" t="n">
-        <v>-124374</v>
+        <v>-582605</v>
       </c>
       <c r="I461" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287921</t>
+          <t>Rechazo PMP1287920</t>
         </is>
       </c>
     </row>
@@ -11076,11 +11072,11 @@
       </c>
       <c r="D462" s="10" t="inlineStr">
         <is>
-          <t>PMP1287928</t>
+          <t>PMP1287921</t>
         </is>
       </c>
       <c r="E462" s="6" t="n">
-        <v>-246230</v>
+        <v>-124374</v>
       </c>
       <c r="F462" s="10" t="inlineStr">
         <is>
@@ -11093,11 +11089,11 @@
         </is>
       </c>
       <c r="H462" s="6" t="n">
-        <v>-246230</v>
+        <v>-124374</v>
       </c>
       <c r="I462" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287928</t>
+          <t>Rechazo PMP1287921</t>
         </is>
       </c>
     </row>
@@ -11109,11 +11105,11 @@
       </c>
       <c r="D463" s="10" t="inlineStr">
         <is>
-          <t>PMP1287930</t>
+          <t>PMP1287928</t>
         </is>
       </c>
       <c r="E463" s="6" t="n">
-        <v>-91079</v>
+        <v>-246230</v>
       </c>
       <c r="F463" s="10" t="inlineStr">
         <is>
@@ -11126,11 +11122,11 @@
         </is>
       </c>
       <c r="H463" s="6" t="n">
-        <v>-91079</v>
+        <v>-246230</v>
       </c>
       <c r="I463" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287930</t>
+          <t>Rechazo PMP1287928</t>
         </is>
       </c>
     </row>
@@ -11142,11 +11138,11 @@
       </c>
       <c r="D464" s="10" t="inlineStr">
         <is>
-          <t>PMP1287931</t>
+          <t>PMP1287930</t>
         </is>
       </c>
       <c r="E464" s="6" t="n">
-        <v>-215025</v>
+        <v>-91079</v>
       </c>
       <c r="F464" s="10" t="inlineStr">
         <is>
@@ -11159,11 +11155,11 @@
         </is>
       </c>
       <c r="H464" s="6" t="n">
-        <v>-215025</v>
+        <v>-91079</v>
       </c>
       <c r="I464" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287931</t>
+          <t>Rechazo PMP1287930</t>
         </is>
       </c>
     </row>
@@ -11175,11 +11171,11 @@
       </c>
       <c r="D465" s="10" t="inlineStr">
         <is>
-          <t>PMP1287948</t>
+          <t>PMP1287931</t>
         </is>
       </c>
       <c r="E465" s="6" t="n">
-        <v>-354871</v>
+        <v>-215025</v>
       </c>
       <c r="F465" s="10" t="inlineStr">
         <is>
@@ -11192,11 +11188,11 @@
         </is>
       </c>
       <c r="H465" s="6" t="n">
-        <v>-354871</v>
+        <v>-215025</v>
       </c>
       <c r="I465" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287948</t>
+          <t>Rechazo PMP1287931</t>
         </is>
       </c>
     </row>
@@ -11208,11 +11204,11 @@
       </c>
       <c r="D466" s="10" t="inlineStr">
         <is>
-          <t>PMP1287949</t>
+          <t>PMP1287948</t>
         </is>
       </c>
       <c r="E466" s="6" t="n">
-        <v>-410669</v>
+        <v>-354871</v>
       </c>
       <c r="F466" s="10" t="inlineStr">
         <is>
@@ -11225,11 +11221,11 @@
         </is>
       </c>
       <c r="H466" s="6" t="n">
-        <v>-410669</v>
+        <v>-354871</v>
       </c>
       <c r="I466" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287949</t>
+          <t>Rechazo PMP1287948</t>
         </is>
       </c>
     </row>
@@ -11241,11 +11237,11 @@
       </c>
       <c r="D467" s="10" t="inlineStr">
         <is>
-          <t>PMP1287951</t>
+          <t>PMP1287949</t>
         </is>
       </c>
       <c r="E467" s="6" t="n">
-        <v>-29456389</v>
+        <v>-410669</v>
       </c>
       <c r="F467" s="10" t="inlineStr">
         <is>
@@ -11258,11 +11254,11 @@
         </is>
       </c>
       <c r="H467" s="6" t="n">
-        <v>-29456389</v>
+        <v>-410669</v>
       </c>
       <c r="I467" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287951</t>
+          <t>Rechazo PMP1287949</t>
         </is>
       </c>
     </row>
@@ -11274,11 +11270,11 @@
       </c>
       <c r="D468" s="10" t="inlineStr">
         <is>
-          <t>PMP1287957</t>
+          <t>PMP1287951</t>
         </is>
       </c>
       <c r="E468" s="6" t="n">
-        <v>-107492</v>
+        <v>-29456389</v>
       </c>
       <c r="F468" s="10" t="inlineStr">
         <is>
@@ -11291,11 +11287,11 @@
         </is>
       </c>
       <c r="H468" s="6" t="n">
-        <v>-107492</v>
+        <v>-29456389</v>
       </c>
       <c r="I468" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287957</t>
+          <t>Rechazo PMP1287951</t>
         </is>
       </c>
     </row>
@@ -11307,11 +11303,11 @@
       </c>
       <c r="D469" s="10" t="inlineStr">
         <is>
-          <t>PMP1288418</t>
+          <t>PMP1287957</t>
         </is>
       </c>
       <c r="E469" s="6" t="n">
-        <v>-2183651</v>
+        <v>-107492</v>
       </c>
       <c r="F469" s="10" t="inlineStr">
         <is>
@@ -11324,11 +11320,11 @@
         </is>
       </c>
       <c r="H469" s="6" t="n">
-        <v>-2183651</v>
+        <v>-107492</v>
       </c>
       <c r="I469" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288418</t>
+          <t>Rechazo PMP1287957</t>
         </is>
       </c>
     </row>
@@ -11340,11 +11336,11 @@
       </c>
       <c r="D470" s="10" t="inlineStr">
         <is>
-          <t>PMP1288731</t>
+          <t>PMP1288418</t>
         </is>
       </c>
       <c r="E470" s="6" t="n">
-        <v>-160222</v>
+        <v>-2183651</v>
       </c>
       <c r="F470" s="10" t="inlineStr">
         <is>
@@ -11357,11 +11353,11 @@
         </is>
       </c>
       <c r="H470" s="6" t="n">
-        <v>-160222</v>
+        <v>-2183651</v>
       </c>
       <c r="I470" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288731</t>
+          <t>Rechazo PMP1288418</t>
         </is>
       </c>
     </row>
@@ -11373,11 +11369,11 @@
       </c>
       <c r="D471" s="10" t="inlineStr">
         <is>
-          <t>PMP1288919</t>
+          <t>PMP1288731</t>
         </is>
       </c>
       <c r="E471" s="6" t="n">
-        <v>-9852</v>
+        <v>-160222</v>
       </c>
       <c r="F471" s="10" t="inlineStr">
         <is>
@@ -11390,11 +11386,11 @@
         </is>
       </c>
       <c r="H471" s="6" t="n">
-        <v>-9852</v>
+        <v>-160222</v>
       </c>
       <c r="I471" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288919</t>
+          <t>Rechazo PMP1288731</t>
         </is>
       </c>
     </row>
@@ -11406,11 +11402,11 @@
       </c>
       <c r="D472" s="10" t="inlineStr">
         <is>
-          <t>PMP1288926</t>
+          <t>PMP1288919</t>
         </is>
       </c>
       <c r="E472" s="6" t="n">
-        <v>-322749</v>
+        <v>-9852</v>
       </c>
       <c r="F472" s="10" t="inlineStr">
         <is>
@@ -11423,11 +11419,11 @@
         </is>
       </c>
       <c r="H472" s="6" t="n">
-        <v>-322749</v>
+        <v>-9852</v>
       </c>
       <c r="I472" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288926</t>
+          <t>Rechazo PMP1288919</t>
         </is>
       </c>
     </row>
@@ -11439,11 +11435,11 @@
       </c>
       <c r="D473" s="10" t="inlineStr">
         <is>
-          <t>PMP1288987</t>
+          <t>PMP1288926</t>
         </is>
       </c>
       <c r="E473" s="6" t="n">
-        <v>-1106307</v>
+        <v>-322749</v>
       </c>
       <c r="F473" s="10" t="inlineStr">
         <is>
@@ -11456,11 +11452,11 @@
         </is>
       </c>
       <c r="H473" s="6" t="n">
-        <v>-1106307</v>
+        <v>-322749</v>
       </c>
       <c r="I473" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288987</t>
+          <t>Rechazo PMP1288926</t>
         </is>
       </c>
     </row>
@@ -11472,11 +11468,11 @@
       </c>
       <c r="D474" s="10" t="inlineStr">
         <is>
-          <t>PMP1288988</t>
+          <t>PMP1288987</t>
         </is>
       </c>
       <c r="E474" s="6" t="n">
-        <v>-33894</v>
+        <v>-1106307</v>
       </c>
       <c r="F474" s="10" t="inlineStr">
         <is>
@@ -11489,11 +11485,11 @@
         </is>
       </c>
       <c r="H474" s="6" t="n">
-        <v>-33894</v>
+        <v>-1106307</v>
       </c>
       <c r="I474" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288988</t>
+          <t>Rechazo PMP1288987</t>
         </is>
       </c>
     </row>
@@ -11505,11 +11501,11 @@
       </c>
       <c r="D475" s="10" t="inlineStr">
         <is>
-          <t>PMP1288989</t>
+          <t>PMP1288988</t>
         </is>
       </c>
       <c r="E475" s="6" t="n">
-        <v>-2259163</v>
+        <v>-33894</v>
       </c>
       <c r="F475" s="10" t="inlineStr">
         <is>
@@ -11522,11 +11518,11 @@
         </is>
       </c>
       <c r="H475" s="6" t="n">
-        <v>-2259163</v>
+        <v>-33894</v>
       </c>
       <c r="I475" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288989</t>
+          <t>Rechazo PMP1288988</t>
         </is>
       </c>
     </row>
@@ -11538,11 +11534,11 @@
       </c>
       <c r="D476" s="10" t="inlineStr">
         <is>
-          <t>PMP1289251</t>
+          <t>PMP1288989</t>
         </is>
       </c>
       <c r="E476" s="6" t="n">
-        <v>-200703</v>
+        <v>-2259163</v>
       </c>
       <c r="F476" s="10" t="inlineStr">
         <is>
@@ -11555,11 +11551,11 @@
         </is>
       </c>
       <c r="H476" s="6" t="n">
-        <v>-200703</v>
+        <v>-2259163</v>
       </c>
       <c r="I476" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289251</t>
+          <t>Rechazo PMP1288989</t>
         </is>
       </c>
     </row>
@@ -11571,11 +11567,11 @@
       </c>
       <c r="D477" s="10" t="inlineStr">
         <is>
-          <t>PMP1289253</t>
+          <t>PMP1289251</t>
         </is>
       </c>
       <c r="E477" s="6" t="n">
-        <v>-2482097</v>
+        <v>-200703</v>
       </c>
       <c r="F477" s="10" t="inlineStr">
         <is>
@@ -11588,11 +11584,11 @@
         </is>
       </c>
       <c r="H477" s="6" t="n">
-        <v>-2482097</v>
+        <v>-200703</v>
       </c>
       <c r="I477" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289253</t>
+          <t>Rechazo PMP1289251</t>
         </is>
       </c>
     </row>
@@ -11604,11 +11600,11 @@
       </c>
       <c r="D478" s="10" t="inlineStr">
         <is>
-          <t>PMP1289324</t>
+          <t>PMP1289253</t>
         </is>
       </c>
       <c r="E478" s="6" t="n">
-        <v>-532656</v>
+        <v>-2482097</v>
       </c>
       <c r="F478" s="10" t="inlineStr">
         <is>
@@ -11621,11 +11617,11 @@
         </is>
       </c>
       <c r="H478" s="6" t="n">
-        <v>-532656</v>
+        <v>-2482097</v>
       </c>
       <c r="I478" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289324</t>
+          <t>Rechazo PMP1289253</t>
         </is>
       </c>
     </row>
@@ -11637,11 +11633,11 @@
       </c>
       <c r="D479" s="10" t="inlineStr">
         <is>
-          <t>PMP1289326</t>
+          <t>PMP1289324</t>
         </is>
       </c>
       <c r="E479" s="6" t="n">
-        <v>-523796</v>
+        <v>-532656</v>
       </c>
       <c r="F479" s="10" t="inlineStr">
         <is>
@@ -11654,11 +11650,11 @@
         </is>
       </c>
       <c r="H479" s="6" t="n">
-        <v>-523796</v>
+        <v>-532656</v>
       </c>
       <c r="I479" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289326</t>
+          <t>Rechazo PMP1289324</t>
         </is>
       </c>
     </row>
@@ -11670,11 +11666,11 @@
       </c>
       <c r="D480" s="10" t="inlineStr">
         <is>
-          <t>PMP1289328</t>
+          <t>PMP1289326</t>
         </is>
       </c>
       <c r="E480" s="6" t="n">
-        <v>-303757</v>
+        <v>-523796</v>
       </c>
       <c r="F480" s="10" t="inlineStr">
         <is>
@@ -11687,11 +11683,11 @@
         </is>
       </c>
       <c r="H480" s="6" t="n">
-        <v>-303757</v>
+        <v>-523796</v>
       </c>
       <c r="I480" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289328</t>
+          <t>Rechazo PMP1289326</t>
         </is>
       </c>
     </row>
@@ -11703,11 +11699,11 @@
       </c>
       <c r="D481" s="10" t="inlineStr">
         <is>
-          <t>PMP1289507</t>
+          <t>PMP1289328</t>
         </is>
       </c>
       <c r="E481" s="6" t="n">
-        <v>-160184</v>
+        <v>-303757</v>
       </c>
       <c r="F481" s="10" t="inlineStr">
         <is>
@@ -11720,11 +11716,11 @@
         </is>
       </c>
       <c r="H481" s="6" t="n">
-        <v>-160184</v>
+        <v>-303757</v>
       </c>
       <c r="I481" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289507</t>
+          <t>Rechazo PMP1289328</t>
         </is>
       </c>
     </row>
@@ -11736,26 +11732,59 @@
       </c>
       <c r="D482" s="10" t="inlineStr">
         <is>
+          <t>PMP1289507</t>
+        </is>
+      </c>
+      <c r="E482" s="6" t="n">
+        <v>-160184</v>
+      </c>
+      <c r="F482" s="10" t="inlineStr">
+        <is>
+          <t>Rechazo</t>
+        </is>
+      </c>
+      <c r="G482" s="10" t="inlineStr">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="H482" s="6" t="n">
+        <v>-160184</v>
+      </c>
+      <c r="I482" s="11" t="inlineStr">
+        <is>
+          <t>Rechazo PMP1289507</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="C483" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D483" s="10" t="inlineStr">
+        <is>
           <t>Costo de Transferen</t>
         </is>
       </c>
-      <c r="E482" s="6" t="n">
+      <c r="E483" s="6" t="n">
         <v>-3000</v>
       </c>
-      <c r="F482" s="10" t="inlineStr">
+      <c r="F483" s="10" t="inlineStr">
         <is>
           <t>Costo de Transferen</t>
         </is>
       </c>
-      <c r="G482" s="10" t="inlineStr">
+      <c r="G483" s="10" t="inlineStr">
         <is>
           <t>WOB</t>
         </is>
       </c>
-      <c r="H482" s="6" t="n">
+      <c r="H483" s="6" t="n">
         <v>-3000</v>
       </c>
-      <c r="I482" s="11" t="inlineStr">
+      <c r="I483" s="11" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>

</xml_diff>

<commit_message>
Ajuste en comentario Cenco, y otrden de template
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_Cenco.xlsx
@@ -583,7 +583,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>01/12/2025</t>
+          <t>02/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8003,28 +8003,28 @@
       </c>
       <c r="D369" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO APERTURA</t>
+          <t>PMP1286553</t>
         </is>
       </c>
       <c r="E369" s="6" t="n">
-        <v>-8594192</v>
+        <v>5910047.02</v>
       </c>
       <c r="F369" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Myr Vlr Pagado</t>
         </is>
       </c>
       <c r="G369" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>388</t>
         </is>
       </c>
       <c r="H369" s="6" t="n">
-        <v>-8594192</v>
+        <v>5910047.02</v>
       </c>
       <c r="I369" s="11" t="inlineStr">
         <is>
-          <t>DAV DSCTO 20.251.100.200.165 DESCUENTO APERTURA DROGUER</t>
+          <t>Myr Vlr Pagado PMP1286553</t>
         </is>
       </c>
     </row>
@@ -8036,28 +8036,28 @@
       </c>
       <c r="D370" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1282099</t>
         </is>
       </c>
       <c r="E370" s="6" t="n">
-        <v>-117913970</v>
+        <v>-307519</v>
       </c>
       <c r="F370" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G370" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H370" s="6" t="n">
-        <v>-117913970</v>
+        <v>-307519</v>
       </c>
       <c r="I370" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.100.199.887 DESCUENTO CALENDARI DROGUER</t>
+          <t>Rechazo PMP1282099</t>
         </is>
       </c>
     </row>
@@ -8069,28 +8069,28 @@
       </c>
       <c r="D371" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1282353</t>
         </is>
       </c>
       <c r="E371" s="6" t="n">
-        <v>-343622707</v>
+        <v>-2659670</v>
       </c>
       <c r="F371" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G371" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H371" s="6" t="n">
-        <v>-343622707</v>
+        <v>-2659670</v>
       </c>
       <c r="I371" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.100.199.918 DESCUENTO CALENDARI DROGUER</t>
+          <t>Rechazo PMP1282353</t>
         </is>
       </c>
     </row>
@@ -8102,28 +8102,28 @@
       </c>
       <c r="D372" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1282964</t>
         </is>
       </c>
       <c r="E372" s="6" t="n">
-        <v>-272000000</v>
+        <v>-185365</v>
       </c>
       <c r="F372" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G372" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H372" s="6" t="n">
-        <v>-272000000</v>
+        <v>-185365</v>
       </c>
       <c r="I372" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.100.199.957 DESCUENTO CALENDARI DROGUER</t>
+          <t>Rechazo PMP1282964</t>
         </is>
       </c>
     </row>
@@ -8135,28 +8135,28 @@
       </c>
       <c r="D373" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1283008</t>
         </is>
       </c>
       <c r="E373" s="6" t="n">
-        <v>-63971913</v>
+        <v>-9788</v>
       </c>
       <c r="F373" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G373" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H373" s="6" t="n">
-        <v>-63971913</v>
+        <v>-9788</v>
       </c>
       <c r="I373" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.100.200.097 DESCUENTO CALENDARI DROGUER</t>
+          <t>Rechazo PMP1283008</t>
         </is>
       </c>
     </row>
@@ -8168,28 +8168,28 @@
       </c>
       <c r="D374" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1283012</t>
         </is>
       </c>
       <c r="E374" s="6" t="n">
-        <v>-20000000</v>
+        <v>-167913</v>
       </c>
       <c r="F374" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G374" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H374" s="6" t="n">
-        <v>-20000000</v>
+        <v>-167913</v>
       </c>
       <c r="I374" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.100.200.166 DESCUENTO CALENDARI DROGUER</t>
+          <t>Rechazo PMP1283012</t>
         </is>
       </c>
     </row>
@@ -8201,28 +8201,28 @@
       </c>
       <c r="D375" s="10" t="inlineStr">
         <is>
-          <t>DEVOLUCIONES</t>
+          <t>PMP1283476</t>
         </is>
       </c>
       <c r="E375" s="6" t="n">
-        <v>-3354641</v>
+        <v>-836339</v>
       </c>
       <c r="F375" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G375" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H375" s="6" t="n">
-        <v>-3354641</v>
+        <v>-836339</v>
       </c>
       <c r="I375" s="11" t="inlineStr">
         <is>
-          <t>DND DSCTO 20.171.100.014.225 DEVOLUCIONES DROGUER</t>
+          <t>Rechazo PMP1283476</t>
         </is>
       </c>
     </row>
@@ -8234,28 +8234,28 @@
       </c>
       <c r="D376" s="10" t="inlineStr">
         <is>
-          <t>DEVOLUCIONES</t>
+          <t>PMP1283500</t>
         </is>
       </c>
       <c r="E376" s="6" t="n">
-        <v>-157710</v>
+        <v>-473742856</v>
       </c>
       <c r="F376" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G376" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H376" s="6" t="n">
-        <v>-157710</v>
+        <v>-473742856</v>
       </c>
       <c r="I376" s="11" t="inlineStr">
         <is>
-          <t>DND DSCTO 20.181.100.045.651 DEVOLUCIONES DROGUER</t>
+          <t>Rechazo PMP1283500</t>
         </is>
       </c>
     </row>
@@ -8267,28 +8267,28 @@
       </c>
       <c r="D377" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>PMP1283784</t>
         </is>
       </c>
       <c r="E377" s="6" t="n">
-        <v>-39137474</v>
+        <v>-629893</v>
       </c>
       <c r="F377" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G377" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H377" s="6" t="n">
-        <v>-39137474</v>
+        <v>-629893</v>
       </c>
       <c r="I377" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO 20.171.100.014.225 DSTO COMERCIAL FIJO DROGUER</t>
+          <t>Rechazo PMP1283784</t>
         </is>
       </c>
     </row>
@@ -8300,28 +8300,28 @@
       </c>
       <c r="D378" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>PMP1283785</t>
         </is>
       </c>
       <c r="E378" s="6" t="n">
-        <v>-6254394</v>
+        <v>-160273</v>
       </c>
       <c r="F378" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G378" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H378" s="6" t="n">
-        <v>-6254394</v>
+        <v>-160273</v>
       </c>
       <c r="I378" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO 20.181.100.032.054 DSTO COMERCIAL FIJO DROGUER</t>
+          <t>Rechazo PMP1283785</t>
         </is>
       </c>
     </row>
@@ -8333,28 +8333,28 @@
       </c>
       <c r="D379" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>PMP1284114</t>
         </is>
       </c>
       <c r="E379" s="6" t="n">
-        <v>-2891340</v>
+        <v>-764103</v>
       </c>
       <c r="F379" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G379" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H379" s="6" t="n">
-        <v>-2891340</v>
+        <v>-764103</v>
       </c>
       <c r="I379" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO 20.181.100.045.651 DSTO COMERCIAL FIJO DROGUER</t>
+          <t>Rechazo PMP1284114</t>
         </is>
       </c>
     </row>
@@ -8366,28 +8366,28 @@
       </c>
       <c r="D380" s="10" t="inlineStr">
         <is>
-          <t>DTO POR ESCALA VOLU</t>
+          <t>PMP1284117</t>
         </is>
       </c>
       <c r="E380" s="6" t="n">
-        <v>-69868245</v>
+        <v>-177051</v>
       </c>
       <c r="F380" s="10" t="inlineStr">
         <is>
-          <t>DROGUER</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G380" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H380" s="6" t="n">
-        <v>-69868245</v>
+        <v>-177051</v>
       </c>
       <c r="I380" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20.251.100.199.283 DTO POR ESCALA VOLU DROGUER</t>
+          <t>Rechazo PMP1284117</t>
         </is>
       </c>
     </row>
@@ -8399,28 +8399,28 @@
       </c>
       <c r="D381" s="10" t="inlineStr">
         <is>
-          <t>VPP1 2004529</t>
+          <t>PMP1284119</t>
         </is>
       </c>
       <c r="E381" s="6" t="n">
-        <v>-57239000</v>
+        <v>-644997</v>
       </c>
       <c r="F381" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEED</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G381" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H381" s="6" t="n">
-        <v>-57239000</v>
+        <v>-644997</v>
       </c>
       <c r="I381" s="11" t="inlineStr">
         <is>
-          <t>VPP1 2004529</t>
+          <t>Rechazo PMP1284119</t>
         </is>
       </c>
     </row>
@@ -8432,28 +8432,28 @@
       </c>
       <c r="D382" s="10" t="inlineStr">
         <is>
-          <t>VPP1 2004621</t>
+          <t>PMP1284200</t>
         </is>
       </c>
       <c r="E382" s="6" t="n">
-        <v>-6426000</v>
+        <v>-175153</v>
       </c>
       <c r="F382" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEED</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G382" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H382" s="6" t="n">
-        <v>-6426000</v>
+        <v>-175153</v>
       </c>
       <c r="I382" s="11" t="inlineStr">
         <is>
-          <t>VPP1 2004621</t>
+          <t>Rechazo PMP1284200</t>
         </is>
       </c>
     </row>
@@ -8465,28 +8465,28 @@
       </c>
       <c r="D383" s="10" t="inlineStr">
         <is>
-          <t>VPP1 2004622</t>
+          <t>PMP1284460</t>
         </is>
       </c>
       <c r="E383" s="6" t="n">
-        <v>-41650000</v>
+        <v>-167879</v>
       </c>
       <c r="F383" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEED</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G383" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H383" s="6" t="n">
-        <v>-41650000</v>
+        <v>-167879</v>
       </c>
       <c r="I383" s="11" t="inlineStr">
         <is>
-          <t>VPP1 2004622</t>
+          <t>Rechazo PMP1284460</t>
         </is>
       </c>
     </row>
@@ -8498,28 +8498,28 @@
       </c>
       <c r="D384" s="10" t="inlineStr">
         <is>
-          <t>VPP2 2021716</t>
+          <t>PMP1284462</t>
         </is>
       </c>
       <c r="E384" s="6" t="n">
-        <v>-2507098292</v>
+        <v>-322931</v>
       </c>
       <c r="F384" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEED</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G384" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H384" s="6" t="n">
-        <v>-2507098292</v>
+        <v>-322931</v>
       </c>
       <c r="I384" s="11" t="inlineStr">
         <is>
-          <t>VPP2 2021716</t>
+          <t>Rechazo PMP1284462</t>
         </is>
       </c>
     </row>
@@ -8531,28 +8531,28 @@
       </c>
       <c r="D385" s="10" t="inlineStr">
         <is>
-          <t>VPP2 2022342</t>
+          <t>PMP1284529</t>
         </is>
       </c>
       <c r="E385" s="6" t="n">
-        <v>-1075965191</v>
+        <v>-276742</v>
       </c>
       <c r="F385" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEED</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G385" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H385" s="6" t="n">
-        <v>-1075965191</v>
+        <v>-276742</v>
       </c>
       <c r="I385" s="11" t="inlineStr">
         <is>
-          <t>VPP2 2022342</t>
+          <t>Rechazo PMP1284529</t>
         </is>
       </c>
     </row>
@@ -8564,28 +8564,28 @@
       </c>
       <c r="D386" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>PMP1284543</t>
         </is>
       </c>
       <c r="E386" s="6" t="n">
-        <v>-37.26000004360685</v>
+        <v>-3015665</v>
       </c>
       <c r="F386" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G386" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H386" s="6" t="n">
-        <v>-37.26000004360685</v>
+        <v>-3015665</v>
       </c>
       <c r="I386" s="11" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Rechazo PMP1284543</t>
         </is>
       </c>
     </row>
@@ -8597,28 +8597,28 @@
       </c>
       <c r="D387" s="10" t="inlineStr">
         <is>
-          <t>PMP1286054</t>
+          <t>PMP1284546</t>
         </is>
       </c>
       <c r="E387" s="6" t="n">
-        <v>-864163</v>
+        <v>-135409</v>
       </c>
       <c r="F387" s="10" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G387" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H387" s="6" t="n">
-        <v>-864163</v>
+        <v>-135409</v>
       </c>
       <c r="I387" s="11" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado PMP1286054</t>
+          <t>Rechazo PMP1284546</t>
         </is>
       </c>
     </row>
@@ -8630,28 +8630,28 @@
       </c>
       <c r="D388" s="10" t="inlineStr">
         <is>
-          <t>PMP1286550</t>
+          <t>PMP1284602</t>
         </is>
       </c>
       <c r="E388" s="6" t="n">
-        <v>-5910046.859999999</v>
+        <v>-930108</v>
       </c>
       <c r="F388" s="10" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G388" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H388" s="6" t="n">
-        <v>-5910046.859999999</v>
+        <v>-930108</v>
       </c>
       <c r="I388" s="11" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado PMP1286550</t>
+          <t>Rechazo PMP1284602</t>
         </is>
       </c>
     </row>
@@ -8663,28 +8663,28 @@
       </c>
       <c r="D389" s="10" t="inlineStr">
         <is>
-          <t>PMP1286553</t>
+          <t>PMP1284750</t>
         </is>
       </c>
       <c r="E389" s="6" t="n">
-        <v>5910047.02</v>
+        <v>-405708</v>
       </c>
       <c r="F389" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G389" s="10" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H389" s="6" t="n">
-        <v>5910047.02</v>
+        <v>-405708</v>
       </c>
       <c r="I389" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1286553</t>
+          <t>Rechazo PMP1284750</t>
         </is>
       </c>
     </row>
@@ -8696,28 +8696,28 @@
       </c>
       <c r="D390" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO APERTURA</t>
+          <t>PMP1284800</t>
         </is>
       </c>
       <c r="E390" s="6" t="n">
-        <v>-14258141</v>
+        <v>-635980</v>
       </c>
       <c r="F390" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G390" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H390" s="6" t="n">
-        <v>-14258141</v>
+        <v>-635980</v>
       </c>
       <c r="I390" s="11" t="inlineStr">
         <is>
-          <t>DAV DSCTO 20.251.200.200.056 DESCUENTO APERTURA PERFUME</t>
+          <t>Rechazo PMP1284800</t>
         </is>
       </c>
     </row>
@@ -8729,28 +8729,28 @@
       </c>
       <c r="D391" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1284876</t>
         </is>
       </c>
       <c r="E391" s="6" t="n">
-        <v>-408729662</v>
+        <v>-689804</v>
       </c>
       <c r="F391" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G391" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H391" s="6" t="n">
-        <v>-408729662</v>
+        <v>-689804</v>
       </c>
       <c r="I391" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.200.199.218 DESCUENTO CALENDARI PERFUME</t>
+          <t>Rechazo PMP1284876</t>
         </is>
       </c>
     </row>
@@ -8762,28 +8762,28 @@
       </c>
       <c r="D392" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1284878</t>
         </is>
       </c>
       <c r="E392" s="6" t="n">
-        <v>-532175699</v>
+        <v>-135533</v>
       </c>
       <c r="F392" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G392" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H392" s="6" t="n">
-        <v>-532175699</v>
+        <v>-135533</v>
       </c>
       <c r="I392" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.200.199.219 DESCUENTO CALENDARI PERFUME</t>
+          <t>Rechazo PMP1284878</t>
         </is>
       </c>
     </row>
@@ -8795,28 +8795,28 @@
       </c>
       <c r="D393" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1284879</t>
         </is>
       </c>
       <c r="E393" s="6" t="n">
-        <v>-542708897</v>
+        <v>-732728</v>
       </c>
       <c r="F393" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G393" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H393" s="6" t="n">
-        <v>-542708897</v>
+        <v>-732728</v>
       </c>
       <c r="I393" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.200.199.221 DESCUENTO CALENDARI PERFUME</t>
+          <t>Rechazo PMP1284879</t>
         </is>
       </c>
     </row>
@@ -8828,28 +8828,28 @@
       </c>
       <c r="D394" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1284948</t>
         </is>
       </c>
       <c r="E394" s="6" t="n">
-        <v>-1323072</v>
+        <v>-1060968</v>
       </c>
       <c r="F394" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G394" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H394" s="6" t="n">
-        <v>-1323072</v>
+        <v>-1060968</v>
       </c>
       <c r="I394" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.200.199.280 DESCUENTO CALENDARI PERFUME</t>
+          <t>Rechazo PMP1284948</t>
         </is>
       </c>
     </row>
@@ -8861,28 +8861,28 @@
       </c>
       <c r="D395" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1284949</t>
         </is>
       </c>
       <c r="E395" s="6" t="n">
-        <v>-254331040</v>
+        <v>-215248</v>
       </c>
       <c r="F395" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G395" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H395" s="6" t="n">
-        <v>-254331040</v>
+        <v>-215248</v>
       </c>
       <c r="I395" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.200.200.036 DESCUENTO CALENDARI PERFUME</t>
+          <t>Rechazo PMP1284949</t>
         </is>
       </c>
     </row>
@@ -8894,28 +8894,28 @@
       </c>
       <c r="D396" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1284950</t>
         </is>
       </c>
       <c r="E396" s="6" t="n">
-        <v>-19632788</v>
+        <v>-1297475</v>
       </c>
       <c r="F396" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G396" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H396" s="6" t="n">
-        <v>-19632788</v>
+        <v>-1297475</v>
       </c>
       <c r="I396" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.200.200.064 DESCUENTO CALENDARI PERFUME</t>
+          <t>Rechazo PMP1284950</t>
         </is>
       </c>
     </row>
@@ -8927,28 +8927,28 @@
       </c>
       <c r="D397" s="10" t="inlineStr">
         <is>
-          <t>DEVOLUCIONES</t>
+          <t>PMP1284951</t>
         </is>
       </c>
       <c r="E397" s="6" t="n">
-        <v>-2074733</v>
+        <v>-5702098</v>
       </c>
       <c r="F397" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G397" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H397" s="6" t="n">
-        <v>-2074733</v>
+        <v>-5702098</v>
       </c>
       <c r="I397" s="11" t="inlineStr">
         <is>
-          <t>DND DSCTO 20.171.200.014.220 DEVOLUCIONES PERFUME</t>
+          <t>Rechazo PMP1284951</t>
         </is>
       </c>
     </row>
@@ -8960,28 +8960,28 @@
       </c>
       <c r="D398" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>PMP1285048</t>
         </is>
       </c>
       <c r="E398" s="6" t="n">
-        <v>-48410423</v>
+        <v>-221603</v>
       </c>
       <c r="F398" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G398" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H398" s="6" t="n">
-        <v>-48410423</v>
+        <v>-221603</v>
       </c>
       <c r="I398" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO 20.171.200.014.220 DSTO COMERCIAL FIJO PERFUME</t>
+          <t>Rechazo PMP1285048</t>
         </is>
       </c>
     </row>
@@ -8993,28 +8993,28 @@
       </c>
       <c r="D399" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>PMP1285059</t>
         </is>
       </c>
       <c r="E399" s="6" t="n">
-        <v>-28246208</v>
+        <v>-160294</v>
       </c>
       <c r="F399" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G399" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H399" s="6" t="n">
-        <v>-28246208</v>
+        <v>-160294</v>
       </c>
       <c r="I399" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO 20.181.200.033.536 DSTO COMERCIAL FIJO PERFUME</t>
+          <t>Rechazo PMP1285059</t>
         </is>
       </c>
     </row>
@@ -9026,28 +9026,28 @@
       </c>
       <c r="D400" s="10" t="inlineStr">
         <is>
-          <t>DTO POR ESCALA VOLU</t>
+          <t>PMP1285065</t>
         </is>
       </c>
       <c r="E400" s="6" t="n">
-        <v>-128010036</v>
+        <v>-107552</v>
       </c>
       <c r="F400" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G400" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H400" s="6" t="n">
-        <v>-128010036</v>
+        <v>-107552</v>
       </c>
       <c r="I400" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20.251.200.199.299 DTO POR ESCALA VOLU PERFUME</t>
+          <t>Rechazo PMP1285065</t>
         </is>
       </c>
     </row>
@@ -9059,28 +9059,28 @@
       </c>
       <c r="D401" s="10" t="inlineStr">
         <is>
-          <t>DTO POR ESCALA VOLU</t>
+          <t>PMP1285067</t>
         </is>
       </c>
       <c r="E401" s="6" t="n">
-        <v>-29342807</v>
+        <v>-135307</v>
       </c>
       <c r="F401" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G401" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H401" s="6" t="n">
-        <v>-29342807</v>
+        <v>-135307</v>
       </c>
       <c r="I401" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20.251.200.199.300 DTO POR ESCALA VOLU PERFUME</t>
+          <t>Rechazo PMP1285067</t>
         </is>
       </c>
     </row>
@@ -9092,28 +9092,28 @@
       </c>
       <c r="D402" s="10" t="inlineStr">
         <is>
-          <t>DTO POR ESCALA VOLU</t>
+          <t>PMP1285071</t>
         </is>
       </c>
       <c r="E402" s="6" t="n">
-        <v>-1719421</v>
+        <v>-419436</v>
       </c>
       <c r="F402" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G402" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H402" s="6" t="n">
-        <v>-1719421</v>
+        <v>-419436</v>
       </c>
       <c r="I402" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20.251.200.199.301 DTO POR ESCALA VOLU PERFUME</t>
+          <t>Rechazo PMP1285071</t>
         </is>
       </c>
     </row>
@@ -9125,28 +9125,28 @@
       </c>
       <c r="D403" s="10" t="inlineStr">
         <is>
-          <t>DTO POR ESCALA VOLU</t>
+          <t>PMP1285653</t>
         </is>
       </c>
       <c r="E403" s="6" t="n">
-        <v>-10000000</v>
+        <v>-558246</v>
       </c>
       <c r="F403" s="10" t="inlineStr">
         <is>
-          <t>PERFUME</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G403" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H403" s="6" t="n">
-        <v>-10000000</v>
+        <v>-558246</v>
       </c>
       <c r="I403" s="11" t="inlineStr">
         <is>
-          <t>DEC DSCTO 20.251.200.200.041 DTO POR ESCALA VOLU PERFUME</t>
+          <t>Rechazo PMP1285653</t>
         </is>
       </c>
     </row>
@@ -9158,28 +9158,28 @@
       </c>
       <c r="D404" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1285659</t>
         </is>
       </c>
       <c r="E404" s="6" t="n">
-        <v>-2074459</v>
+        <v>-311765</v>
       </c>
       <c r="F404" s="10" t="inlineStr">
         <is>
-          <t>PLATOS</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G404" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H404" s="6" t="n">
-        <v>-2074459</v>
+        <v>-311765</v>
       </c>
       <c r="I404" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.222.600.126.372 DESCUENTO CALENDARI PLATOS</t>
+          <t>Rechazo PMP1285659</t>
         </is>
       </c>
     </row>
@@ -9191,28 +9191,28 @@
       </c>
       <c r="D405" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1285725</t>
         </is>
       </c>
       <c r="E405" s="6" t="n">
-        <v>-11353075</v>
+        <v>-679290</v>
       </c>
       <c r="F405" s="10" t="inlineStr">
         <is>
-          <t>PLATOS</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G405" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H405" s="6" t="n">
-        <v>-11353075</v>
+        <v>-679290</v>
       </c>
       <c r="I405" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.252.600.198.821 DESCUENTO CALENDARI PLATOS</t>
+          <t>Rechazo PMP1285725</t>
         </is>
       </c>
     </row>
@@ -9224,28 +9224,28 @@
       </c>
       <c r="D406" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO COMPRAS</t>
+          <t>PMP1285898</t>
         </is>
       </c>
       <c r="E406" s="6" t="n">
-        <v>-1394767</v>
+        <v>-253685</v>
       </c>
       <c r="F406" s="10" t="inlineStr">
         <is>
-          <t>PLATOS</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G406" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H406" s="6" t="n">
-        <v>-1394767</v>
+        <v>-253685</v>
       </c>
       <c r="I406" s="11" t="inlineStr">
         <is>
-          <t>DCC DSCTO 20.222.600.126.372 DESCUENTO COMPRAS PLATOS</t>
+          <t>Rechazo PMP1285898</t>
         </is>
       </c>
     </row>
@@ -9257,28 +9257,28 @@
       </c>
       <c r="D407" s="10" t="inlineStr">
         <is>
-          <t>DSTO COMERCIAL FIJO</t>
+          <t>PMP1285903</t>
         </is>
       </c>
       <c r="E407" s="6" t="n">
-        <v>-20921503</v>
+        <v>-322554</v>
       </c>
       <c r="F407" s="10" t="inlineStr">
         <is>
-          <t>PLATOS</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G407" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H407" s="6" t="n">
-        <v>-20921503</v>
+        <v>-322554</v>
       </c>
       <c r="I407" s="11" t="inlineStr">
         <is>
-          <t>DCF DSCTO 20.222.600.126.372 DSTO COMERCIAL FIJO PLATOS</t>
+          <t>Rechazo PMP1285903</t>
         </is>
       </c>
     </row>
@@ -9290,28 +9290,28 @@
       </c>
       <c r="D408" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO CALENDARI</t>
+          <t>PMP1285908</t>
         </is>
       </c>
       <c r="E408" s="6" t="n">
-        <v>-29638456</v>
+        <v>-135255</v>
       </c>
       <c r="F408" s="10" t="inlineStr">
         <is>
-          <t>RANCHO</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G408" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H408" s="6" t="n">
-        <v>-29638456</v>
+        <v>-135255</v>
       </c>
       <c r="I408" s="11" t="inlineStr">
         <is>
-          <t>DCA DSCTO 20.251.400.199.149 DESCUENTO CALENDARI RANCHO</t>
+          <t>Rechazo PMP1285908</t>
         </is>
       </c>
     </row>
@@ -9323,28 +9323,28 @@
       </c>
       <c r="D409" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO COMERCIAL</t>
+          <t>PMP1286056</t>
         </is>
       </c>
       <c r="E409" s="6" t="n">
-        <v>-61299192</v>
+        <v>-556413</v>
       </c>
       <c r="F409" s="10" t="inlineStr">
         <is>
-          <t>RANCHO</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G409" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H409" s="6" t="n">
-        <v>-61299192</v>
+        <v>-556413</v>
       </c>
       <c r="I409" s="11" t="inlineStr">
         <is>
-          <t>RPL DSCTO 0 DESCUENTO COMERCIAL RANCHO</t>
+          <t>Rechazo PMP1286056</t>
         </is>
       </c>
     </row>
@@ -9356,28 +9356,28 @@
       </c>
       <c r="D410" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO EN PRIMER</t>
+          <t>PMP1286208</t>
         </is>
       </c>
       <c r="E410" s="6" t="n">
-        <v>-10216531</v>
+        <v>-949123</v>
       </c>
       <c r="F410" s="10" t="inlineStr">
         <is>
-          <t>RANCHO</t>
+          <t>Rechazo</t>
         </is>
       </c>
       <c r="G410" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H410" s="6" t="n">
-        <v>-10216531</v>
+        <v>-949123</v>
       </c>
       <c r="I410" s="11" t="inlineStr">
         <is>
-          <t>DPC DSCTO 0 DESCUENTO EN PRIMER RANCHO</t>
+          <t>Rechazo PMP1286208</t>
         </is>
       </c>
     </row>
@@ -9389,11 +9389,11 @@
       </c>
       <c r="D411" s="10" t="inlineStr">
         <is>
-          <t>PMP1282099</t>
+          <t>PMP1286554</t>
         </is>
       </c>
       <c r="E411" s="6" t="n">
-        <v>-307519</v>
+        <v>-354934</v>
       </c>
       <c r="F411" s="10" t="inlineStr">
         <is>
@@ -9406,11 +9406,11 @@
         </is>
       </c>
       <c r="H411" s="6" t="n">
-        <v>-307519</v>
+        <v>-354934</v>
       </c>
       <c r="I411" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1282099</t>
+          <t>Rechazo PMP1286554</t>
         </is>
       </c>
     </row>
@@ -9422,11 +9422,11 @@
       </c>
       <c r="D412" s="10" t="inlineStr">
         <is>
-          <t>PMP1282353</t>
+          <t>PMP1286556</t>
         </is>
       </c>
       <c r="E412" s="6" t="n">
-        <v>-2659670</v>
+        <v>-364001</v>
       </c>
       <c r="F412" s="10" t="inlineStr">
         <is>
@@ -9439,11 +9439,11 @@
         </is>
       </c>
       <c r="H412" s="6" t="n">
-        <v>-2659670</v>
+        <v>-364001</v>
       </c>
       <c r="I412" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1282353</t>
+          <t>Rechazo PMP1286556</t>
         </is>
       </c>
     </row>
@@ -9455,11 +9455,11 @@
       </c>
       <c r="D413" s="10" t="inlineStr">
         <is>
-          <t>PMP1282964</t>
+          <t>PMP1286709</t>
         </is>
       </c>
       <c r="E413" s="6" t="n">
-        <v>-185365</v>
+        <v>-33537478</v>
       </c>
       <c r="F413" s="10" t="inlineStr">
         <is>
@@ -9472,11 +9472,11 @@
         </is>
       </c>
       <c r="H413" s="6" t="n">
-        <v>-185365</v>
+        <v>-33537478</v>
       </c>
       <c r="I413" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1282964</t>
+          <t>Rechazo PMP1286709</t>
         </is>
       </c>
     </row>
@@ -9488,11 +9488,11 @@
       </c>
       <c r="D414" s="10" t="inlineStr">
         <is>
-          <t>PMP1283008</t>
+          <t>PMP1286710</t>
         </is>
       </c>
       <c r="E414" s="6" t="n">
-        <v>-9788</v>
+        <v>-650618</v>
       </c>
       <c r="F414" s="10" t="inlineStr">
         <is>
@@ -9505,11 +9505,11 @@
         </is>
       </c>
       <c r="H414" s="6" t="n">
-        <v>-9788</v>
+        <v>-650618</v>
       </c>
       <c r="I414" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283008</t>
+          <t>Rechazo PMP1286710</t>
         </is>
       </c>
     </row>
@@ -9521,11 +9521,11 @@
       </c>
       <c r="D415" s="10" t="inlineStr">
         <is>
-          <t>PMP1283012</t>
+          <t>PMP1286711</t>
         </is>
       </c>
       <c r="E415" s="6" t="n">
-        <v>-167913</v>
+        <v>-6920570</v>
       </c>
       <c r="F415" s="10" t="inlineStr">
         <is>
@@ -9538,11 +9538,11 @@
         </is>
       </c>
       <c r="H415" s="6" t="n">
-        <v>-167913</v>
+        <v>-6920570</v>
       </c>
       <c r="I415" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283012</t>
+          <t>Rechazo PMP1286711</t>
         </is>
       </c>
     </row>
@@ -9554,11 +9554,11 @@
       </c>
       <c r="D416" s="10" t="inlineStr">
         <is>
-          <t>PMP1283476</t>
+          <t>PMP1286712</t>
         </is>
       </c>
       <c r="E416" s="6" t="n">
-        <v>-836339</v>
+        <v>-403395</v>
       </c>
       <c r="F416" s="10" t="inlineStr">
         <is>
@@ -9571,11 +9571,11 @@
         </is>
       </c>
       <c r="H416" s="6" t="n">
-        <v>-836339</v>
+        <v>-403395</v>
       </c>
       <c r="I416" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283476</t>
+          <t>Rechazo PMP1286712</t>
         </is>
       </c>
     </row>
@@ -9587,11 +9587,11 @@
       </c>
       <c r="D417" s="10" t="inlineStr">
         <is>
-          <t>PMP1283500</t>
+          <t>PMP1286715</t>
         </is>
       </c>
       <c r="E417" s="6" t="n">
-        <v>-473742856</v>
+        <v>-4085189</v>
       </c>
       <c r="F417" s="10" t="inlineStr">
         <is>
@@ -9604,11 +9604,11 @@
         </is>
       </c>
       <c r="H417" s="6" t="n">
-        <v>-473742856</v>
+        <v>-4085189</v>
       </c>
       <c r="I417" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283500</t>
+          <t>Rechazo PMP1286715</t>
         </is>
       </c>
     </row>
@@ -9620,11 +9620,11 @@
       </c>
       <c r="D418" s="10" t="inlineStr">
         <is>
-          <t>PMP1283784</t>
+          <t>PMP1286716</t>
         </is>
       </c>
       <c r="E418" s="6" t="n">
-        <v>-629893</v>
+        <v>-822039</v>
       </c>
       <c r="F418" s="10" t="inlineStr">
         <is>
@@ -9637,11 +9637,11 @@
         </is>
       </c>
       <c r="H418" s="6" t="n">
-        <v>-629893</v>
+        <v>-822039</v>
       </c>
       <c r="I418" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283784</t>
+          <t>Rechazo PMP1286716</t>
         </is>
       </c>
     </row>
@@ -9653,11 +9653,11 @@
       </c>
       <c r="D419" s="10" t="inlineStr">
         <is>
-          <t>PMP1283785</t>
+          <t>PMP1287257</t>
         </is>
       </c>
       <c r="E419" s="6" t="n">
-        <v>-160273</v>
+        <v>-156625</v>
       </c>
       <c r="F419" s="10" t="inlineStr">
         <is>
@@ -9670,11 +9670,11 @@
         </is>
       </c>
       <c r="H419" s="6" t="n">
-        <v>-160273</v>
+        <v>-156625</v>
       </c>
       <c r="I419" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1283785</t>
+          <t>Rechazo PMP1287257</t>
         </is>
       </c>
     </row>
@@ -9686,11 +9686,11 @@
       </c>
       <c r="D420" s="10" t="inlineStr">
         <is>
-          <t>PMP1284114</t>
+          <t>PMP1287321</t>
         </is>
       </c>
       <c r="E420" s="6" t="n">
-        <v>-764103</v>
+        <v>-182163</v>
       </c>
       <c r="F420" s="10" t="inlineStr">
         <is>
@@ -9703,11 +9703,11 @@
         </is>
       </c>
       <c r="H420" s="6" t="n">
-        <v>-764103</v>
+        <v>-182163</v>
       </c>
       <c r="I420" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284114</t>
+          <t>Rechazo PMP1287321</t>
         </is>
       </c>
     </row>
@@ -9719,11 +9719,11 @@
       </c>
       <c r="D421" s="10" t="inlineStr">
         <is>
-          <t>PMP1284117</t>
+          <t>PMP1287325</t>
         </is>
       </c>
       <c r="E421" s="6" t="n">
-        <v>-177051</v>
+        <v>-118625</v>
       </c>
       <c r="F421" s="10" t="inlineStr">
         <is>
@@ -9736,11 +9736,11 @@
         </is>
       </c>
       <c r="H421" s="6" t="n">
-        <v>-177051</v>
+        <v>-118625</v>
       </c>
       <c r="I421" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284117</t>
+          <t>Rechazo PMP1287325</t>
         </is>
       </c>
     </row>
@@ -9752,11 +9752,11 @@
       </c>
       <c r="D422" s="10" t="inlineStr">
         <is>
-          <t>PMP1284119</t>
+          <t>PMP1287335</t>
         </is>
       </c>
       <c r="E422" s="6" t="n">
-        <v>-644997</v>
+        <v>-128620</v>
       </c>
       <c r="F422" s="10" t="inlineStr">
         <is>
@@ -9769,11 +9769,11 @@
         </is>
       </c>
       <c r="H422" s="6" t="n">
-        <v>-644997</v>
+        <v>-128620</v>
       </c>
       <c r="I422" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284119</t>
+          <t>Rechazo PMP1287335</t>
         </is>
       </c>
     </row>
@@ -9785,11 +9785,11 @@
       </c>
       <c r="D423" s="10" t="inlineStr">
         <is>
-          <t>PMP1284200</t>
+          <t>PMP1287379</t>
         </is>
       </c>
       <c r="E423" s="6" t="n">
-        <v>-175153</v>
+        <v>-271757</v>
       </c>
       <c r="F423" s="10" t="inlineStr">
         <is>
@@ -9802,11 +9802,11 @@
         </is>
       </c>
       <c r="H423" s="6" t="n">
-        <v>-175153</v>
+        <v>-271757</v>
       </c>
       <c r="I423" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284200</t>
+          <t>Rechazo PMP1287379</t>
         </is>
       </c>
     </row>
@@ -9818,11 +9818,11 @@
       </c>
       <c r="D424" s="10" t="inlineStr">
         <is>
-          <t>PMP1284460</t>
+          <t>PMP1287385</t>
         </is>
       </c>
       <c r="E424" s="6" t="n">
-        <v>-167879</v>
+        <v>-214996</v>
       </c>
       <c r="F424" s="10" t="inlineStr">
         <is>
@@ -9835,11 +9835,11 @@
         </is>
       </c>
       <c r="H424" s="6" t="n">
-        <v>-167879</v>
+        <v>-214996</v>
       </c>
       <c r="I424" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284460</t>
+          <t>Rechazo PMP1287385</t>
         </is>
       </c>
     </row>
@@ -9851,11 +9851,11 @@
       </c>
       <c r="D425" s="10" t="inlineStr">
         <is>
-          <t>PMP1284462</t>
+          <t>PMP1287386</t>
         </is>
       </c>
       <c r="E425" s="6" t="n">
-        <v>-322931</v>
+        <v>-267680</v>
       </c>
       <c r="F425" s="10" t="inlineStr">
         <is>
@@ -9868,11 +9868,11 @@
         </is>
       </c>
       <c r="H425" s="6" t="n">
-        <v>-322931</v>
+        <v>-267680</v>
       </c>
       <c r="I425" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284462</t>
+          <t>Rechazo PMP1287386</t>
         </is>
       </c>
     </row>
@@ -9884,11 +9884,11 @@
       </c>
       <c r="D426" s="10" t="inlineStr">
         <is>
-          <t>PMP1284529</t>
+          <t>PMP1287574</t>
         </is>
       </c>
       <c r="E426" s="6" t="n">
-        <v>-276742</v>
+        <v>-11940004</v>
       </c>
       <c r="F426" s="10" t="inlineStr">
         <is>
@@ -9901,11 +9901,11 @@
         </is>
       </c>
       <c r="H426" s="6" t="n">
-        <v>-276742</v>
+        <v>-11940004</v>
       </c>
       <c r="I426" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284529</t>
+          <t>Rechazo PMP1287574</t>
         </is>
       </c>
     </row>
@@ -9917,11 +9917,11 @@
       </c>
       <c r="D427" s="10" t="inlineStr">
         <is>
-          <t>PMP1284543</t>
+          <t>PMP1287736</t>
         </is>
       </c>
       <c r="E427" s="6" t="n">
-        <v>-3015665</v>
+        <v>-93440</v>
       </c>
       <c r="F427" s="10" t="inlineStr">
         <is>
@@ -9934,11 +9934,11 @@
         </is>
       </c>
       <c r="H427" s="6" t="n">
-        <v>-3015665</v>
+        <v>-93440</v>
       </c>
       <c r="I427" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284543</t>
+          <t>Rechazo PMP1287736</t>
         </is>
       </c>
     </row>
@@ -9950,11 +9950,11 @@
       </c>
       <c r="D428" s="10" t="inlineStr">
         <is>
-          <t>PMP1284546</t>
+          <t>PMP128777746</t>
         </is>
       </c>
       <c r="E428" s="6" t="n">
-        <v>-135409</v>
+        <v>-322500</v>
       </c>
       <c r="F428" s="10" t="inlineStr">
         <is>
@@ -9967,11 +9967,11 @@
         </is>
       </c>
       <c r="H428" s="6" t="n">
-        <v>-135409</v>
+        <v>-322500</v>
       </c>
       <c r="I428" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284546</t>
+          <t>Rechazo PMP128777746</t>
         </is>
       </c>
     </row>
@@ -9983,11 +9983,11 @@
       </c>
       <c r="D429" s="10" t="inlineStr">
         <is>
-          <t>PMP1284602</t>
+          <t>PMP1287829</t>
         </is>
       </c>
       <c r="E429" s="6" t="n">
-        <v>-930108</v>
+        <v>-290823</v>
       </c>
       <c r="F429" s="10" t="inlineStr">
         <is>
@@ -10000,11 +10000,11 @@
         </is>
       </c>
       <c r="H429" s="6" t="n">
-        <v>-930108</v>
+        <v>-290823</v>
       </c>
       <c r="I429" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284602</t>
+          <t>Rechazo PMP1287829</t>
         </is>
       </c>
     </row>
@@ -10016,11 +10016,11 @@
       </c>
       <c r="D430" s="10" t="inlineStr">
         <is>
-          <t>PMP1284750</t>
+          <t>PMP1287903</t>
         </is>
       </c>
       <c r="E430" s="6" t="n">
-        <v>-405708</v>
+        <v>-128514</v>
       </c>
       <c r="F430" s="10" t="inlineStr">
         <is>
@@ -10033,11 +10033,11 @@
         </is>
       </c>
       <c r="H430" s="6" t="n">
-        <v>-405708</v>
+        <v>-128514</v>
       </c>
       <c r="I430" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284750</t>
+          <t>Rechazo PMP1287903</t>
         </is>
       </c>
     </row>
@@ -10049,11 +10049,11 @@
       </c>
       <c r="D431" s="10" t="inlineStr">
         <is>
-          <t>PMP1284800</t>
+          <t>PMP1287904</t>
         </is>
       </c>
       <c r="E431" s="6" t="n">
-        <v>-635980</v>
+        <v>-80064</v>
       </c>
       <c r="F431" s="10" t="inlineStr">
         <is>
@@ -10066,11 +10066,11 @@
         </is>
       </c>
       <c r="H431" s="6" t="n">
-        <v>-635980</v>
+        <v>-80064</v>
       </c>
       <c r="I431" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284800</t>
+          <t>Rechazo PMP1287904</t>
         </is>
       </c>
     </row>
@@ -10082,11 +10082,11 @@
       </c>
       <c r="D432" s="10" t="inlineStr">
         <is>
-          <t>PMP1284876</t>
+          <t>PMP1287920</t>
         </is>
       </c>
       <c r="E432" s="6" t="n">
-        <v>-689804</v>
+        <v>-582605</v>
       </c>
       <c r="F432" s="10" t="inlineStr">
         <is>
@@ -10099,11 +10099,11 @@
         </is>
       </c>
       <c r="H432" s="6" t="n">
-        <v>-689804</v>
+        <v>-582605</v>
       </c>
       <c r="I432" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284876</t>
+          <t>Rechazo PMP1287920</t>
         </is>
       </c>
     </row>
@@ -10115,11 +10115,11 @@
       </c>
       <c r="D433" s="10" t="inlineStr">
         <is>
-          <t>PMP1284878</t>
+          <t>PMP1287921</t>
         </is>
       </c>
       <c r="E433" s="6" t="n">
-        <v>-135533</v>
+        <v>-124374</v>
       </c>
       <c r="F433" s="10" t="inlineStr">
         <is>
@@ -10132,11 +10132,11 @@
         </is>
       </c>
       <c r="H433" s="6" t="n">
-        <v>-135533</v>
+        <v>-124374</v>
       </c>
       <c r="I433" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284878</t>
+          <t>Rechazo PMP1287921</t>
         </is>
       </c>
     </row>
@@ -10148,11 +10148,11 @@
       </c>
       <c r="D434" s="10" t="inlineStr">
         <is>
-          <t>PMP1284879</t>
+          <t>PMP1287928</t>
         </is>
       </c>
       <c r="E434" s="6" t="n">
-        <v>-732728</v>
+        <v>-246230</v>
       </c>
       <c r="F434" s="10" t="inlineStr">
         <is>
@@ -10165,11 +10165,11 @@
         </is>
       </c>
       <c r="H434" s="6" t="n">
-        <v>-732728</v>
+        <v>-246230</v>
       </c>
       <c r="I434" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284879</t>
+          <t>Rechazo PMP1287928</t>
         </is>
       </c>
     </row>
@@ -10181,11 +10181,11 @@
       </c>
       <c r="D435" s="10" t="inlineStr">
         <is>
-          <t>PMP1284948</t>
+          <t>PMP1287930</t>
         </is>
       </c>
       <c r="E435" s="6" t="n">
-        <v>-1060968</v>
+        <v>-91079</v>
       </c>
       <c r="F435" s="10" t="inlineStr">
         <is>
@@ -10198,11 +10198,11 @@
         </is>
       </c>
       <c r="H435" s="6" t="n">
-        <v>-1060968</v>
+        <v>-91079</v>
       </c>
       <c r="I435" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284948</t>
+          <t>Rechazo PMP1287930</t>
         </is>
       </c>
     </row>
@@ -10214,11 +10214,11 @@
       </c>
       <c r="D436" s="10" t="inlineStr">
         <is>
-          <t>PMP1284949</t>
+          <t>PMP1287931</t>
         </is>
       </c>
       <c r="E436" s="6" t="n">
-        <v>-215248</v>
+        <v>-215025</v>
       </c>
       <c r="F436" s="10" t="inlineStr">
         <is>
@@ -10231,11 +10231,11 @@
         </is>
       </c>
       <c r="H436" s="6" t="n">
-        <v>-215248</v>
+        <v>-215025</v>
       </c>
       <c r="I436" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284949</t>
+          <t>Rechazo PMP1287931</t>
         </is>
       </c>
     </row>
@@ -10247,11 +10247,11 @@
       </c>
       <c r="D437" s="10" t="inlineStr">
         <is>
-          <t>PMP1284950</t>
+          <t>PMP1287948</t>
         </is>
       </c>
       <c r="E437" s="6" t="n">
-        <v>-1297475</v>
+        <v>-354871</v>
       </c>
       <c r="F437" s="10" t="inlineStr">
         <is>
@@ -10264,11 +10264,11 @@
         </is>
       </c>
       <c r="H437" s="6" t="n">
-        <v>-1297475</v>
+        <v>-354871</v>
       </c>
       <c r="I437" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284950</t>
+          <t>Rechazo PMP1287948</t>
         </is>
       </c>
     </row>
@@ -10280,11 +10280,11 @@
       </c>
       <c r="D438" s="10" t="inlineStr">
         <is>
-          <t>PMP1284951</t>
+          <t>PMP1287949</t>
         </is>
       </c>
       <c r="E438" s="6" t="n">
-        <v>-5702098</v>
+        <v>-410669</v>
       </c>
       <c r="F438" s="10" t="inlineStr">
         <is>
@@ -10297,11 +10297,11 @@
         </is>
       </c>
       <c r="H438" s="6" t="n">
-        <v>-5702098</v>
+        <v>-410669</v>
       </c>
       <c r="I438" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1284951</t>
+          <t>Rechazo PMP1287949</t>
         </is>
       </c>
     </row>
@@ -10313,11 +10313,11 @@
       </c>
       <c r="D439" s="10" t="inlineStr">
         <is>
-          <t>PMP1285048</t>
+          <t>PMP1287951</t>
         </is>
       </c>
       <c r="E439" s="6" t="n">
-        <v>-221603</v>
+        <v>-29456389</v>
       </c>
       <c r="F439" s="10" t="inlineStr">
         <is>
@@ -10330,11 +10330,11 @@
         </is>
       </c>
       <c r="H439" s="6" t="n">
-        <v>-221603</v>
+        <v>-29456389</v>
       </c>
       <c r="I439" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285048</t>
+          <t>Rechazo PMP1287951</t>
         </is>
       </c>
     </row>
@@ -10346,11 +10346,11 @@
       </c>
       <c r="D440" s="10" t="inlineStr">
         <is>
-          <t>PMP1285059</t>
+          <t>PMP1287957</t>
         </is>
       </c>
       <c r="E440" s="6" t="n">
-        <v>-160294</v>
+        <v>-107492</v>
       </c>
       <c r="F440" s="10" t="inlineStr">
         <is>
@@ -10363,11 +10363,11 @@
         </is>
       </c>
       <c r="H440" s="6" t="n">
-        <v>-160294</v>
+        <v>-107492</v>
       </c>
       <c r="I440" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285059</t>
+          <t>Rechazo PMP1287957</t>
         </is>
       </c>
     </row>
@@ -10379,11 +10379,11 @@
       </c>
       <c r="D441" s="10" t="inlineStr">
         <is>
-          <t>PMP1285065</t>
+          <t>PMP1288418</t>
         </is>
       </c>
       <c r="E441" s="6" t="n">
-        <v>-107552</v>
+        <v>-2183651</v>
       </c>
       <c r="F441" s="10" t="inlineStr">
         <is>
@@ -10396,11 +10396,11 @@
         </is>
       </c>
       <c r="H441" s="6" t="n">
-        <v>-107552</v>
+        <v>-2183651</v>
       </c>
       <c r="I441" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285065</t>
+          <t>Rechazo PMP1288418</t>
         </is>
       </c>
     </row>
@@ -10412,11 +10412,11 @@
       </c>
       <c r="D442" s="10" t="inlineStr">
         <is>
-          <t>PMP1285067</t>
+          <t>PMP1288731</t>
         </is>
       </c>
       <c r="E442" s="6" t="n">
-        <v>-135307</v>
+        <v>-160222</v>
       </c>
       <c r="F442" s="10" t="inlineStr">
         <is>
@@ -10429,11 +10429,11 @@
         </is>
       </c>
       <c r="H442" s="6" t="n">
-        <v>-135307</v>
+        <v>-160222</v>
       </c>
       <c r="I442" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285067</t>
+          <t>Rechazo PMP1288731</t>
         </is>
       </c>
     </row>
@@ -10445,11 +10445,11 @@
       </c>
       <c r="D443" s="10" t="inlineStr">
         <is>
-          <t>PMP1285071</t>
+          <t>PMP1288919</t>
         </is>
       </c>
       <c r="E443" s="6" t="n">
-        <v>-419436</v>
+        <v>-9852</v>
       </c>
       <c r="F443" s="10" t="inlineStr">
         <is>
@@ -10462,11 +10462,11 @@
         </is>
       </c>
       <c r="H443" s="6" t="n">
-        <v>-419436</v>
+        <v>-9852</v>
       </c>
       <c r="I443" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285071</t>
+          <t>Rechazo PMP1288919</t>
         </is>
       </c>
     </row>
@@ -10478,11 +10478,11 @@
       </c>
       <c r="D444" s="10" t="inlineStr">
         <is>
-          <t>PMP1285653</t>
+          <t>PMP1288926</t>
         </is>
       </c>
       <c r="E444" s="6" t="n">
-        <v>-558246</v>
+        <v>-322749</v>
       </c>
       <c r="F444" s="10" t="inlineStr">
         <is>
@@ -10495,11 +10495,11 @@
         </is>
       </c>
       <c r="H444" s="6" t="n">
-        <v>-558246</v>
+        <v>-322749</v>
       </c>
       <c r="I444" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285653</t>
+          <t>Rechazo PMP1288926</t>
         </is>
       </c>
     </row>
@@ -10511,11 +10511,11 @@
       </c>
       <c r="D445" s="10" t="inlineStr">
         <is>
-          <t>PMP1285659</t>
+          <t>PMP1288987</t>
         </is>
       </c>
       <c r="E445" s="6" t="n">
-        <v>-311765</v>
+        <v>-1106307</v>
       </c>
       <c r="F445" s="10" t="inlineStr">
         <is>
@@ -10528,11 +10528,11 @@
         </is>
       </c>
       <c r="H445" s="6" t="n">
-        <v>-311765</v>
+        <v>-1106307</v>
       </c>
       <c r="I445" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285659</t>
+          <t>Rechazo PMP1288987</t>
         </is>
       </c>
     </row>
@@ -10544,11 +10544,11 @@
       </c>
       <c r="D446" s="10" t="inlineStr">
         <is>
-          <t>PMP1285725</t>
+          <t>PMP1288988</t>
         </is>
       </c>
       <c r="E446" s="6" t="n">
-        <v>-679290</v>
+        <v>-33894</v>
       </c>
       <c r="F446" s="10" t="inlineStr">
         <is>
@@ -10561,11 +10561,11 @@
         </is>
       </c>
       <c r="H446" s="6" t="n">
-        <v>-679290</v>
+        <v>-33894</v>
       </c>
       <c r="I446" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285725</t>
+          <t>Rechazo PMP1288988</t>
         </is>
       </c>
     </row>
@@ -10577,11 +10577,11 @@
       </c>
       <c r="D447" s="10" t="inlineStr">
         <is>
-          <t>PMP1285898</t>
+          <t>PMP1288989</t>
         </is>
       </c>
       <c r="E447" s="6" t="n">
-        <v>-253685</v>
+        <v>-2259163</v>
       </c>
       <c r="F447" s="10" t="inlineStr">
         <is>
@@ -10594,11 +10594,11 @@
         </is>
       </c>
       <c r="H447" s="6" t="n">
-        <v>-253685</v>
+        <v>-2259163</v>
       </c>
       <c r="I447" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285898</t>
+          <t>Rechazo PMP1288989</t>
         </is>
       </c>
     </row>
@@ -10610,11 +10610,11 @@
       </c>
       <c r="D448" s="10" t="inlineStr">
         <is>
-          <t>PMP1285903</t>
+          <t>PMP1289251</t>
         </is>
       </c>
       <c r="E448" s="6" t="n">
-        <v>-322554</v>
+        <v>-200703</v>
       </c>
       <c r="F448" s="10" t="inlineStr">
         <is>
@@ -10627,11 +10627,11 @@
         </is>
       </c>
       <c r="H448" s="6" t="n">
-        <v>-322554</v>
+        <v>-200703</v>
       </c>
       <c r="I448" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285903</t>
+          <t>Rechazo PMP1289251</t>
         </is>
       </c>
     </row>
@@ -10643,11 +10643,11 @@
       </c>
       <c r="D449" s="10" t="inlineStr">
         <is>
-          <t>PMP1285908</t>
+          <t>PMP1289253</t>
         </is>
       </c>
       <c r="E449" s="6" t="n">
-        <v>-135255</v>
+        <v>-2482097</v>
       </c>
       <c r="F449" s="10" t="inlineStr">
         <is>
@@ -10660,11 +10660,11 @@
         </is>
       </c>
       <c r="H449" s="6" t="n">
-        <v>-135255</v>
+        <v>-2482097</v>
       </c>
       <c r="I449" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1285908</t>
+          <t>Rechazo PMP1289253</t>
         </is>
       </c>
     </row>
@@ -10676,11 +10676,11 @@
       </c>
       <c r="D450" s="10" t="inlineStr">
         <is>
-          <t>PMP1286056</t>
+          <t>PMP1289324</t>
         </is>
       </c>
       <c r="E450" s="6" t="n">
-        <v>-556413</v>
+        <v>-532656</v>
       </c>
       <c r="F450" s="10" t="inlineStr">
         <is>
@@ -10693,11 +10693,11 @@
         </is>
       </c>
       <c r="H450" s="6" t="n">
-        <v>-556413</v>
+        <v>-532656</v>
       </c>
       <c r="I450" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286056</t>
+          <t>Rechazo PMP1289324</t>
         </is>
       </c>
     </row>
@@ -10709,11 +10709,11 @@
       </c>
       <c r="D451" s="10" t="inlineStr">
         <is>
-          <t>PMP1286208</t>
+          <t>PMP1289326</t>
         </is>
       </c>
       <c r="E451" s="6" t="n">
-        <v>-949123</v>
+        <v>-523796</v>
       </c>
       <c r="F451" s="10" t="inlineStr">
         <is>
@@ -10726,11 +10726,11 @@
         </is>
       </c>
       <c r="H451" s="6" t="n">
-        <v>-949123</v>
+        <v>-523796</v>
       </c>
       <c r="I451" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286208</t>
+          <t>Rechazo PMP1289326</t>
         </is>
       </c>
     </row>
@@ -10742,11 +10742,11 @@
       </c>
       <c r="D452" s="10" t="inlineStr">
         <is>
-          <t>PMP1286554</t>
+          <t>PMP1289328</t>
         </is>
       </c>
       <c r="E452" s="6" t="n">
-        <v>-354934</v>
+        <v>-303757</v>
       </c>
       <c r="F452" s="10" t="inlineStr">
         <is>
@@ -10759,11 +10759,11 @@
         </is>
       </c>
       <c r="H452" s="6" t="n">
-        <v>-354934</v>
+        <v>-303757</v>
       </c>
       <c r="I452" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286554</t>
+          <t>Rechazo PMP1289328</t>
         </is>
       </c>
     </row>
@@ -10775,11 +10775,11 @@
       </c>
       <c r="D453" s="10" t="inlineStr">
         <is>
-          <t>PMP1286556</t>
+          <t>PMP1289507</t>
         </is>
       </c>
       <c r="E453" s="6" t="n">
-        <v>-364001</v>
+        <v>-160184</v>
       </c>
       <c r="F453" s="10" t="inlineStr">
         <is>
@@ -10792,11 +10792,11 @@
         </is>
       </c>
       <c r="H453" s="6" t="n">
-        <v>-364001</v>
+        <v>-160184</v>
       </c>
       <c r="I453" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286556</t>
+          <t>Rechazo PMP1289507</t>
         </is>
       </c>
     </row>
@@ -10808,28 +10808,28 @@
       </c>
       <c r="D454" s="10" t="inlineStr">
         <is>
-          <t>PMP1286709</t>
+          <t>DESCUENTO APERTURA</t>
         </is>
       </c>
       <c r="E454" s="6" t="n">
-        <v>-33537478</v>
+        <v>-8594192</v>
       </c>
       <c r="F454" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G454" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H454" s="6" t="n">
-        <v>-33537478</v>
+        <v>-8594192</v>
       </c>
       <c r="I454" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286709</t>
+          <t>DAV DSCTO 20.251.100.200.165 DROGUER DESCUENTO APERTURA</t>
         </is>
       </c>
     </row>
@@ -10841,28 +10841,28 @@
       </c>
       <c r="D455" s="10" t="inlineStr">
         <is>
-          <t>PMP1286710</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E455" s="6" t="n">
-        <v>-650618</v>
+        <v>-117913970</v>
       </c>
       <c r="F455" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G455" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H455" s="6" t="n">
-        <v>-650618</v>
+        <v>-117913970</v>
       </c>
       <c r="I455" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286710</t>
+          <t>DCA DSCTO 20.251.100.199.887 DROGUER DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -10874,28 +10874,28 @@
       </c>
       <c r="D456" s="10" t="inlineStr">
         <is>
-          <t>PMP1286711</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E456" s="6" t="n">
-        <v>-6920570</v>
+        <v>-343622707</v>
       </c>
       <c r="F456" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G456" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H456" s="6" t="n">
-        <v>-6920570</v>
+        <v>-343622707</v>
       </c>
       <c r="I456" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286711</t>
+          <t>DCA DSCTO 20.251.100.199.918 DROGUER DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -10907,28 +10907,28 @@
       </c>
       <c r="D457" s="10" t="inlineStr">
         <is>
-          <t>PMP1286712</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E457" s="6" t="n">
-        <v>-403395</v>
+        <v>-272000000</v>
       </c>
       <c r="F457" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G457" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H457" s="6" t="n">
-        <v>-403395</v>
+        <v>-272000000</v>
       </c>
       <c r="I457" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286712</t>
+          <t>DCA DSCTO 20.251.100.199.957 DROGUER DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -10940,28 +10940,28 @@
       </c>
       <c r="D458" s="10" t="inlineStr">
         <is>
-          <t>PMP1286715</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E458" s="6" t="n">
-        <v>-4085189</v>
+        <v>-63971913</v>
       </c>
       <c r="F458" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G458" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H458" s="6" t="n">
-        <v>-4085189</v>
+        <v>-63971913</v>
       </c>
       <c r="I458" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286715</t>
+          <t>DCA DSCTO 20.251.100.200.097 DROGUER DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -10973,28 +10973,28 @@
       </c>
       <c r="D459" s="10" t="inlineStr">
         <is>
-          <t>PMP1286716</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E459" s="6" t="n">
-        <v>-822039</v>
+        <v>-20000000</v>
       </c>
       <c r="F459" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G459" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H459" s="6" t="n">
-        <v>-822039</v>
+        <v>-20000000</v>
       </c>
       <c r="I459" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1286716</t>
+          <t>DCA DSCTO 20.251.100.200.166 DROGUER DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11006,28 +11006,28 @@
       </c>
       <c r="D460" s="10" t="inlineStr">
         <is>
-          <t>PMP1287257</t>
+          <t>DEVOLUCIONES</t>
         </is>
       </c>
       <c r="E460" s="6" t="n">
-        <v>-156625</v>
+        <v>-3354641</v>
       </c>
       <c r="F460" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G460" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H460" s="6" t="n">
-        <v>-156625</v>
+        <v>-3354641</v>
       </c>
       <c r="I460" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287257</t>
+          <t>DND DSCTO 20.171.100.014.225 DROGUER DEVOLUCIONES</t>
         </is>
       </c>
     </row>
@@ -11039,28 +11039,28 @@
       </c>
       <c r="D461" s="10" t="inlineStr">
         <is>
-          <t>PMP1287321</t>
+          <t>DEVOLUCIONES</t>
         </is>
       </c>
       <c r="E461" s="6" t="n">
-        <v>-182163</v>
+        <v>-157710</v>
       </c>
       <c r="F461" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G461" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H461" s="6" t="n">
-        <v>-182163</v>
+        <v>-157710</v>
       </c>
       <c r="I461" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287321</t>
+          <t>DND DSCTO 20.181.100.045.651 DROGUER DEVOLUCIONES</t>
         </is>
       </c>
     </row>
@@ -11072,28 +11072,28 @@
       </c>
       <c r="D462" s="10" t="inlineStr">
         <is>
-          <t>PMP1287325</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E462" s="6" t="n">
-        <v>-118625</v>
+        <v>-39137474</v>
       </c>
       <c r="F462" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G462" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H462" s="6" t="n">
-        <v>-118625</v>
+        <v>-39137474</v>
       </c>
       <c r="I462" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287325</t>
+          <t>DCF DSCTO 20.171.100.014.225 DROGUER DSTO COMERCIAL FIJO</t>
         </is>
       </c>
     </row>
@@ -11105,28 +11105,28 @@
       </c>
       <c r="D463" s="10" t="inlineStr">
         <is>
-          <t>PMP1287335</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E463" s="6" t="n">
-        <v>-128620</v>
+        <v>-6254394</v>
       </c>
       <c r="F463" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G463" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H463" s="6" t="n">
-        <v>-128620</v>
+        <v>-6254394</v>
       </c>
       <c r="I463" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287335</t>
+          <t>DCF DSCTO 20.181.100.032.054 DROGUER DSTO COMERCIAL FIJO</t>
         </is>
       </c>
     </row>
@@ -11138,28 +11138,28 @@
       </c>
       <c r="D464" s="10" t="inlineStr">
         <is>
-          <t>PMP1287379</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E464" s="6" t="n">
-        <v>-271757</v>
+        <v>-2891340</v>
       </c>
       <c r="F464" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G464" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H464" s="6" t="n">
-        <v>-271757</v>
+        <v>-2891340</v>
       </c>
       <c r="I464" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287379</t>
+          <t>DCF DSCTO 20.181.100.045.651 DROGUER DSTO COMERCIAL FIJO</t>
         </is>
       </c>
     </row>
@@ -11171,28 +11171,28 @@
       </c>
       <c r="D465" s="10" t="inlineStr">
         <is>
-          <t>PMP1287385</t>
+          <t>DTO POR ESCALA VOLU</t>
         </is>
       </c>
       <c r="E465" s="6" t="n">
-        <v>-214996</v>
+        <v>-69868245</v>
       </c>
       <c r="F465" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>DROGUER</t>
         </is>
       </c>
       <c r="G465" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H465" s="6" t="n">
-        <v>-214996</v>
+        <v>-69868245</v>
       </c>
       <c r="I465" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287385</t>
+          <t>DEC DSCTO 20.251.100.199.283 DROGUER DTO POR ESCALA VOLU</t>
         </is>
       </c>
     </row>
@@ -11204,28 +11204,28 @@
       </c>
       <c r="D466" s="10" t="inlineStr">
         <is>
-          <t>PMP1287386</t>
+          <t>DESCUENTO APERTURA</t>
         </is>
       </c>
       <c r="E466" s="6" t="n">
-        <v>-267680</v>
+        <v>-14258141</v>
       </c>
       <c r="F466" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G466" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H466" s="6" t="n">
-        <v>-267680</v>
+        <v>-14258141</v>
       </c>
       <c r="I466" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287386</t>
+          <t>DAV DSCTO 20.251.200.200.056 PERFUME DESCUENTO APERTURA</t>
         </is>
       </c>
     </row>
@@ -11237,28 +11237,28 @@
       </c>
       <c r="D467" s="10" t="inlineStr">
         <is>
-          <t>PMP1287574</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E467" s="6" t="n">
-        <v>-11940004</v>
+        <v>-408729662</v>
       </c>
       <c r="F467" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G467" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H467" s="6" t="n">
-        <v>-11940004</v>
+        <v>-408729662</v>
       </c>
       <c r="I467" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287574</t>
+          <t>DCA DSCTO 20.251.200.199.218 PERFUME DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11270,28 +11270,28 @@
       </c>
       <c r="D468" s="10" t="inlineStr">
         <is>
-          <t>PMP1287736</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E468" s="6" t="n">
-        <v>-93440</v>
+        <v>-532175699</v>
       </c>
       <c r="F468" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G468" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H468" s="6" t="n">
-        <v>-93440</v>
+        <v>-532175699</v>
       </c>
       <c r="I468" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287736</t>
+          <t>DCA DSCTO 20.251.200.199.219 PERFUME DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11303,28 +11303,28 @@
       </c>
       <c r="D469" s="10" t="inlineStr">
         <is>
-          <t>PMP128777746</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E469" s="6" t="n">
-        <v>-322500</v>
+        <v>-542708897</v>
       </c>
       <c r="F469" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G469" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H469" s="6" t="n">
-        <v>-322500</v>
+        <v>-542708897</v>
       </c>
       <c r="I469" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP128777746</t>
+          <t>DCA DSCTO 20.251.200.199.221 PERFUME DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11336,28 +11336,28 @@
       </c>
       <c r="D470" s="10" t="inlineStr">
         <is>
-          <t>PMP1287829</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E470" s="6" t="n">
-        <v>-290823</v>
+        <v>-1323072</v>
       </c>
       <c r="F470" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G470" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H470" s="6" t="n">
-        <v>-290823</v>
+        <v>-1323072</v>
       </c>
       <c r="I470" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287829</t>
+          <t>DCA DSCTO 20.251.200.199.280 PERFUME DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11369,28 +11369,28 @@
       </c>
       <c r="D471" s="10" t="inlineStr">
         <is>
-          <t>PMP1287903</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E471" s="6" t="n">
-        <v>-128514</v>
+        <v>-254331040</v>
       </c>
       <c r="F471" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G471" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H471" s="6" t="n">
-        <v>-128514</v>
+        <v>-254331040</v>
       </c>
       <c r="I471" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287903</t>
+          <t>DCA DSCTO 20.251.200.200.036 PERFUME DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11402,28 +11402,28 @@
       </c>
       <c r="D472" s="10" t="inlineStr">
         <is>
-          <t>PMP1287904</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E472" s="6" t="n">
-        <v>-80064</v>
+        <v>-19632788</v>
       </c>
       <c r="F472" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G472" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H472" s="6" t="n">
-        <v>-80064</v>
+        <v>-19632788</v>
       </c>
       <c r="I472" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287904</t>
+          <t>DCA DSCTO 20.251.200.200.064 PERFUME DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11435,28 +11435,28 @@
       </c>
       <c r="D473" s="10" t="inlineStr">
         <is>
-          <t>PMP1287920</t>
+          <t>DEVOLUCIONES</t>
         </is>
       </c>
       <c r="E473" s="6" t="n">
-        <v>-582605</v>
+        <v>-2074733</v>
       </c>
       <c r="F473" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G473" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H473" s="6" t="n">
-        <v>-582605</v>
+        <v>-2074733</v>
       </c>
       <c r="I473" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287920</t>
+          <t>DND DSCTO 20.171.200.014.220 PERFUME DEVOLUCIONES</t>
         </is>
       </c>
     </row>
@@ -11468,28 +11468,28 @@
       </c>
       <c r="D474" s="10" t="inlineStr">
         <is>
-          <t>PMP1287921</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E474" s="6" t="n">
-        <v>-124374</v>
+        <v>-48410423</v>
       </c>
       <c r="F474" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G474" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H474" s="6" t="n">
-        <v>-124374</v>
+        <v>-48410423</v>
       </c>
       <c r="I474" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287921</t>
+          <t>DCF DSCTO 20.171.200.014.220 PERFUME DSTO COMERCIAL FIJO</t>
         </is>
       </c>
     </row>
@@ -11501,28 +11501,28 @@
       </c>
       <c r="D475" s="10" t="inlineStr">
         <is>
-          <t>PMP1287928</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E475" s="6" t="n">
-        <v>-246230</v>
+        <v>-28246208</v>
       </c>
       <c r="F475" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G475" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H475" s="6" t="n">
-        <v>-246230</v>
+        <v>-28246208</v>
       </c>
       <c r="I475" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287928</t>
+          <t>DCF DSCTO 20.181.200.033.536 PERFUME DSTO COMERCIAL FIJO</t>
         </is>
       </c>
     </row>
@@ -11534,28 +11534,28 @@
       </c>
       <c r="D476" s="10" t="inlineStr">
         <is>
-          <t>PMP1287930</t>
+          <t>DTO POR ESCALA VOLU</t>
         </is>
       </c>
       <c r="E476" s="6" t="n">
-        <v>-91079</v>
+        <v>-128010036</v>
       </c>
       <c r="F476" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G476" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H476" s="6" t="n">
-        <v>-91079</v>
+        <v>-128010036</v>
       </c>
       <c r="I476" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287930</t>
+          <t>DEC DSCTO 20.251.200.199.299 PERFUME DTO POR ESCALA VOLU</t>
         </is>
       </c>
     </row>
@@ -11567,28 +11567,28 @@
       </c>
       <c r="D477" s="10" t="inlineStr">
         <is>
-          <t>PMP1287931</t>
+          <t>DTO POR ESCALA VOLU</t>
         </is>
       </c>
       <c r="E477" s="6" t="n">
-        <v>-215025</v>
+        <v>-29342807</v>
       </c>
       <c r="F477" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G477" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H477" s="6" t="n">
-        <v>-215025</v>
+        <v>-29342807</v>
       </c>
       <c r="I477" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287931</t>
+          <t>DEC DSCTO 20.251.200.199.300 PERFUME DTO POR ESCALA VOLU</t>
         </is>
       </c>
     </row>
@@ -11600,28 +11600,28 @@
       </c>
       <c r="D478" s="10" t="inlineStr">
         <is>
-          <t>PMP1287948</t>
+          <t>DTO POR ESCALA VOLU</t>
         </is>
       </c>
       <c r="E478" s="6" t="n">
-        <v>-354871</v>
+        <v>-1719421</v>
       </c>
       <c r="F478" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G478" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H478" s="6" t="n">
-        <v>-354871</v>
+        <v>-1719421</v>
       </c>
       <c r="I478" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287948</t>
+          <t>DEC DSCTO 20.251.200.199.301 PERFUME DTO POR ESCALA VOLU</t>
         </is>
       </c>
     </row>
@@ -11633,28 +11633,28 @@
       </c>
       <c r="D479" s="10" t="inlineStr">
         <is>
-          <t>PMP1287949</t>
+          <t>DTO POR ESCALA VOLU</t>
         </is>
       </c>
       <c r="E479" s="6" t="n">
-        <v>-410669</v>
+        <v>-10000000</v>
       </c>
       <c r="F479" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PERFUME</t>
         </is>
       </c>
       <c r="G479" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H479" s="6" t="n">
-        <v>-410669</v>
+        <v>-10000000</v>
       </c>
       <c r="I479" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287949</t>
+          <t>DEC DSCTO 20.251.200.200.041 PERFUME DTO POR ESCALA VOLU</t>
         </is>
       </c>
     </row>
@@ -11666,28 +11666,28 @@
       </c>
       <c r="D480" s="10" t="inlineStr">
         <is>
-          <t>PMP1287951</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E480" s="6" t="n">
-        <v>-29456389</v>
+        <v>-2074459</v>
       </c>
       <c r="F480" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PLATOS</t>
         </is>
       </c>
       <c r="G480" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H480" s="6" t="n">
-        <v>-29456389</v>
+        <v>-2074459</v>
       </c>
       <c r="I480" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287951</t>
+          <t>DCA DSCTO 20.222.600.126.372 PLATOS DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11699,28 +11699,28 @@
       </c>
       <c r="D481" s="10" t="inlineStr">
         <is>
-          <t>PMP1287957</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E481" s="6" t="n">
-        <v>-107492</v>
+        <v>-11353075</v>
       </c>
       <c r="F481" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PLATOS</t>
         </is>
       </c>
       <c r="G481" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H481" s="6" t="n">
-        <v>-107492</v>
+        <v>-11353075</v>
       </c>
       <c r="I481" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1287957</t>
+          <t>DCA DSCTO 20.252.600.198.821 PLATOS DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11732,28 +11732,28 @@
       </c>
       <c r="D482" s="10" t="inlineStr">
         <is>
-          <t>PMP1288418</t>
+          <t>DESCUENTO COMPRAS</t>
         </is>
       </c>
       <c r="E482" s="6" t="n">
-        <v>-2183651</v>
+        <v>-1394767</v>
       </c>
       <c r="F482" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PLATOS</t>
         </is>
       </c>
       <c r="G482" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H482" s="6" t="n">
-        <v>-2183651</v>
+        <v>-1394767</v>
       </c>
       <c r="I482" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288418</t>
+          <t>DCC DSCTO 20.222.600.126.372 PLATOS DESCUENTO COMPRAS</t>
         </is>
       </c>
     </row>
@@ -11765,28 +11765,28 @@
       </c>
       <c r="D483" s="10" t="inlineStr">
         <is>
-          <t>PMP1288731</t>
+          <t>DSTO COMERCIAL FIJO</t>
         </is>
       </c>
       <c r="E483" s="6" t="n">
-        <v>-160222</v>
+        <v>-20921503</v>
       </c>
       <c r="F483" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>PLATOS</t>
         </is>
       </c>
       <c r="G483" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H483" s="6" t="n">
-        <v>-160222</v>
+        <v>-20921503</v>
       </c>
       <c r="I483" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288731</t>
+          <t>DCF DSCTO 20.222.600.126.372 PLATOS DSTO COMERCIAL FIJO</t>
         </is>
       </c>
     </row>
@@ -11798,28 +11798,28 @@
       </c>
       <c r="D484" s="10" t="inlineStr">
         <is>
-          <t>PMP1288919</t>
+          <t>DESCUENTO CALENDARI</t>
         </is>
       </c>
       <c r="E484" s="6" t="n">
-        <v>-9852</v>
+        <v>-29638456</v>
       </c>
       <c r="F484" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>RANCHO</t>
         </is>
       </c>
       <c r="G484" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H484" s="6" t="n">
-        <v>-9852</v>
+        <v>-29638456</v>
       </c>
       <c r="I484" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288919</t>
+          <t>DCA DSCTO 20.251.400.199.149 RANCHO DESCUENTO CALENDARI</t>
         </is>
       </c>
     </row>
@@ -11831,28 +11831,28 @@
       </c>
       <c r="D485" s="10" t="inlineStr">
         <is>
-          <t>PMP1288926</t>
+          <t>DESCUENTO COMERCIAL</t>
         </is>
       </c>
       <c r="E485" s="6" t="n">
-        <v>-322749</v>
+        <v>-61299192</v>
       </c>
       <c r="F485" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>RANCHO</t>
         </is>
       </c>
       <c r="G485" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H485" s="6" t="n">
-        <v>-322749</v>
+        <v>-61299192</v>
       </c>
       <c r="I485" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288926</t>
+          <t>RPL DSCTO 0 RANCHO DESCUENTO COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -11864,28 +11864,28 @@
       </c>
       <c r="D486" s="10" t="inlineStr">
         <is>
-          <t>PMP1288987</t>
+          <t>DESCUENTO EN PRIMER</t>
         </is>
       </c>
       <c r="E486" s="6" t="n">
-        <v>-1106307</v>
+        <v>-10216531</v>
       </c>
       <c r="F486" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>RANCHO</t>
         </is>
       </c>
       <c r="G486" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H486" s="6" t="n">
-        <v>-1106307</v>
+        <v>-10216531</v>
       </c>
       <c r="I486" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288987</t>
+          <t>DPC DSCTO 0 RANCHO DESCUENTO EN PRIMER</t>
         </is>
       </c>
     </row>
@@ -11897,28 +11897,28 @@
       </c>
       <c r="D487" s="10" t="inlineStr">
         <is>
-          <t>PMP1288988</t>
+          <t>VPP1 2004529</t>
         </is>
       </c>
       <c r="E487" s="6" t="n">
-        <v>-33894</v>
+        <v>-57239000</v>
       </c>
       <c r="F487" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>FACT PROVEED</t>
         </is>
       </c>
       <c r="G487" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H487" s="6" t="n">
-        <v>-33894</v>
+        <v>-57239000</v>
       </c>
       <c r="I487" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288988</t>
+          <t>FACT PROVEED VPP1 2004529</t>
         </is>
       </c>
     </row>
@@ -11930,28 +11930,28 @@
       </c>
       <c r="D488" s="10" t="inlineStr">
         <is>
-          <t>PMP1288989</t>
+          <t>VPP1 2004621</t>
         </is>
       </c>
       <c r="E488" s="6" t="n">
-        <v>-2259163</v>
+        <v>-6426000</v>
       </c>
       <c r="F488" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>FACT PROVEED</t>
         </is>
       </c>
       <c r="G488" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H488" s="6" t="n">
-        <v>-2259163</v>
+        <v>-6426000</v>
       </c>
       <c r="I488" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1288989</t>
+          <t>FACT PROVEED VPP1 2004621</t>
         </is>
       </c>
     </row>
@@ -11963,28 +11963,28 @@
       </c>
       <c r="D489" s="10" t="inlineStr">
         <is>
-          <t>PMP1289251</t>
+          <t>VPP1 2004622</t>
         </is>
       </c>
       <c r="E489" s="6" t="n">
-        <v>-200703</v>
+        <v>-41650000</v>
       </c>
       <c r="F489" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>FACT PROVEED</t>
         </is>
       </c>
       <c r="G489" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H489" s="6" t="n">
-        <v>-200703</v>
+        <v>-41650000</v>
       </c>
       <c r="I489" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289251</t>
+          <t>FACT PROVEED VPP1 2004622</t>
         </is>
       </c>
     </row>
@@ -11996,28 +11996,28 @@
       </c>
       <c r="D490" s="10" t="inlineStr">
         <is>
-          <t>PMP1289253</t>
+          <t>VPP2 2021716</t>
         </is>
       </c>
       <c r="E490" s="6" t="n">
-        <v>-2482097</v>
+        <v>-2507098292</v>
       </c>
       <c r="F490" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>FACT PROVEED</t>
         </is>
       </c>
       <c r="G490" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H490" s="6" t="n">
-        <v>-2482097</v>
+        <v>-2507098292</v>
       </c>
       <c r="I490" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289253</t>
+          <t>FACT PROVEED VPP2 2021716</t>
         </is>
       </c>
     </row>
@@ -12029,28 +12029,28 @@
       </c>
       <c r="D491" s="10" t="inlineStr">
         <is>
-          <t>PMP1289324</t>
+          <t>VPP2 2022342</t>
         </is>
       </c>
       <c r="E491" s="6" t="n">
-        <v>-532656</v>
+        <v>-1075965191</v>
       </c>
       <c r="F491" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>FACT PROVEED</t>
         </is>
       </c>
       <c r="G491" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H491" s="6" t="n">
-        <v>-532656</v>
+        <v>-1075965191</v>
       </c>
       <c r="I491" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289324</t>
+          <t>FACT PROVEED VPP2 2022342</t>
         </is>
       </c>
     </row>
@@ -12062,28 +12062,28 @@
       </c>
       <c r="D492" s="10" t="inlineStr">
         <is>
-          <t>PMP1289326</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E492" s="6" t="n">
-        <v>-523796</v>
+        <v>-37.26000004360685</v>
       </c>
       <c r="F492" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G492" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H492" s="6" t="n">
-        <v>-523796</v>
+        <v>-37.26000004360685</v>
       </c>
       <c r="I492" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289326</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
@@ -12095,28 +12095,28 @@
       </c>
       <c r="D493" s="10" t="inlineStr">
         <is>
-          <t>PMP1289328</t>
+          <t>PMP1286054</t>
         </is>
       </c>
       <c r="E493" s="6" t="n">
-        <v>-303757</v>
+        <v>-864163</v>
       </c>
       <c r="F493" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>Menor Vlr Pagado</t>
         </is>
       </c>
       <c r="G493" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H493" s="6" t="n">
-        <v>-303757</v>
+        <v>-864163</v>
       </c>
       <c r="I493" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289328</t>
+          <t>Menor Vlr Pagado PMP1286054</t>
         </is>
       </c>
     </row>
@@ -12128,28 +12128,28 @@
       </c>
       <c r="D494" s="10" t="inlineStr">
         <is>
-          <t>PMP1289507</t>
+          <t>PMP1286550</t>
         </is>
       </c>
       <c r="E494" s="6" t="n">
-        <v>-160184</v>
+        <v>-5910046.859999999</v>
       </c>
       <c r="F494" s="10" t="inlineStr">
         <is>
-          <t>Rechazo</t>
+          <t>Menor Vlr Pagado</t>
         </is>
       </c>
       <c r="G494" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H494" s="6" t="n">
-        <v>-160184</v>
+        <v>-5910046.859999999</v>
       </c>
       <c r="I494" s="11" t="inlineStr">
         <is>
-          <t>Rechazo PMP1289507</t>
+          <t>Menor Vlr Pagado PMP1286550</t>
         </is>
       </c>
     </row>

</xml_diff>